<commit_message>
Dashboard: order cards by next action, settled at bottom; running balance column
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011kwt7TrQj5DyWSPAGHQ9fr
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -88,12 +88,45 @@
     <t xml:space="preserve">Net P/L to Date</t>
   </si>
   <si>
-    <t xml:space="preserve">Account Balance After</t>
+    <t xml:space="preserve">Running Balance (display order)</t>
   </si>
   <si>
     <t xml:space="preserve">Detail Tab / Notes</t>
   </si>
   <si>
+    <t xml:space="preserve">MLB Sunday Slate (15 games)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACTIVE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tab: MLB Jul 12 · LIVE — 2-5 thru 7, Giants ML remaining</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WNBA Sunday Doubleheader</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tab: WNBA Jul 12 · Sky@Wings 7 ET, Fever@Aces 9 ET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NASCAR Quaker State 400</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tab: NASCAR Jul 12 · race ~7 PM ET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">World Cup 2026 — Final Four</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jul 14-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tab: World Cup 2026 · semis Tue/Wed, final Sun</t>
+  </si>
+  <si>
     <t xml:space="preserve">UFC 329: McGregor vs Holloway 2</t>
   </si>
   <si>
@@ -104,39 +137,6 @@
   </si>
   <si>
     <t xml:space="preserve">Tab: UFC 329 · 6-3, settled Jul 11 · archives Jul 18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">World Cup 2026 — Final Four</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jul 14-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ACTIVE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tab: World Cup 2026 · semis Tue/Wed, final Sun</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MLB Sunday Slate (15 games)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-07-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tab: MLB Jul 12 · 2-5 thru 7 of 8 · Giants ML still live</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NASCAR Quaker State 400</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tab: NASCAR Jul 12 · race ~7 PM ET</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WNBA Sunday Doubleheader</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tab: WNBA Jul 12 · Sky@Wings 7 ET, Fever@Aces 9 ET</t>
   </si>
   <si>
     <t xml:space="preserve">TOTALS</t>
@@ -1160,17 +1160,20 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="13">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
     <numFmt numFmtId="167" formatCode="\$#,##0.00"/>
-    <numFmt numFmtId="168" formatCode="\+0;\-0"/>
-    <numFmt numFmtId="169" formatCode="0"/>
-    <numFmt numFmtId="170" formatCode="0.0%"/>
-    <numFmt numFmtId="171" formatCode="0%"/>
-    <numFmt numFmtId="172" formatCode="0.0&quot; exp. wins&quot;"/>
-    <numFmt numFmtId="173" formatCode="0.0"/>
+    <numFmt numFmtId="168" formatCode="\$#,##0"/>
+    <numFmt numFmtId="169" formatCode="\$#,##0.00"/>
+    <numFmt numFmtId="170" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
+    <numFmt numFmtId="171" formatCode="\+0;\-0"/>
+    <numFmt numFmtId="172" formatCode="0"/>
+    <numFmt numFmtId="173" formatCode="0.0%"/>
+    <numFmt numFmtId="174" formatCode="0%"/>
+    <numFmt numFmtId="175" formatCode="0.0&quot; exp. wins&quot;"/>
+    <numFmt numFmtId="176" formatCode="0.0"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -1251,7 +1254,7 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <color rgb="FF808080"/>
+      <color rgb="FF1B7A3D"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1266,7 +1269,7 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <color rgb="FF1B7A3D"/>
+      <color rgb="FF808080"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1360,14 +1363,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE7E6E6"/>
-        <bgColor rgb="FFE2F0D9"/>
+        <fgColor rgb="FFE2F0D9"/>
+        <bgColor rgb="FFE7E6E6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE2F0D9"/>
-        <bgColor rgb="FFE7E6E6"/>
+        <fgColor rgb="FFE7E6E6"/>
+        <bgColor rgb="FFE2F0D9"/>
       </patternFill>
     </fill>
     <fill>
@@ -1527,19 +1530,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1559,19 +1562,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1639,7 +1642,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1671,11 +1674,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="172" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1695,15 +1698,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="175" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="176" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1719,7 +1722,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1735,7 +1738,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2154,7 +2157,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B16" s="14" t="s">
         <v>22</v>
@@ -2166,168 +2169,168 @@
         <v>24</v>
       </c>
       <c r="E16" s="16" t="n">
+        <f aca="false">SUM('MLB Jul 12'!F7:F14)</f>
+        <v>1000</v>
+      </c>
+      <c r="F16" s="16" t="n">
+        <f aca="false">SUMIF('MLB Jul 12'!I7:I14,"Pending",'MLB Jul 12'!F7:F14)</f>
+        <v>200</v>
+      </c>
+      <c r="G16" s="17" t="n">
+        <f aca="false">SUM('MLB Jul 12'!J7:J14)</f>
+        <v>473.2</v>
+      </c>
+      <c r="H16" s="18" t="n">
+        <f aca="false">SUM('MLB Jul 12'!K7:K14)</f>
+        <v>-326.8</v>
+      </c>
+      <c r="I16" s="19" t="n">
+        <f aca="false">B5+H16</f>
+        <v>4673.2</v>
+      </c>
+      <c r="J16" s="20" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E17" s="16" t="n">
+        <f aca="false">SUM('WNBA Jul 12'!F7:F13)</f>
+        <v>1000</v>
+      </c>
+      <c r="F17" s="16" t="n">
+        <f aca="false">SUMIF('WNBA Jul 12'!I7:I13,"Pending",'WNBA Jul 12'!F7:F13)</f>
+        <v>1000</v>
+      </c>
+      <c r="G17" s="17" t="n">
+        <f aca="false">SUM('WNBA Jul 12'!J7:J13)</f>
+        <v>0</v>
+      </c>
+      <c r="H17" s="18" t="n">
+        <f aca="false">SUM('WNBA Jul 12'!K7:K13)</f>
+        <v>0</v>
+      </c>
+      <c r="I17" s="19" t="n">
+        <f aca="false">I16+H17</f>
+        <v>4673.2</v>
+      </c>
+      <c r="J17" s="20" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E18" s="16" t="n">
+        <f aca="false">SUM('NASCAR Jul 12'!F7:F13)</f>
+        <v>1000</v>
+      </c>
+      <c r="F18" s="16" t="n">
+        <f aca="false">SUMIF('NASCAR Jul 12'!I7:I13,"Pending",'NASCAR Jul 12'!F7:F13)</f>
+        <v>1000</v>
+      </c>
+      <c r="G18" s="17" t="n">
+        <f aca="false">SUM('NASCAR Jul 12'!J7:J13)</f>
+        <v>0</v>
+      </c>
+      <c r="H18" s="18" t="n">
+        <f aca="false">SUM('NASCAR Jul 12'!K7:K13)</f>
+        <v>0</v>
+      </c>
+      <c r="I18" s="19" t="n">
+        <f aca="false">I17+H18</f>
+        <v>4673.2</v>
+      </c>
+      <c r="J18" s="20" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E19" s="16" t="n">
+        <f aca="false">SUM('World Cup 2026'!F7:F13)</f>
+        <v>1000</v>
+      </c>
+      <c r="F19" s="16" t="n">
+        <f aca="false">SUMIF('World Cup 2026'!I7:I13,"Pending",'World Cup 2026'!F7:F13)</f>
+        <v>1000</v>
+      </c>
+      <c r="G19" s="17" t="n">
+        <f aca="false">SUM('World Cup 2026'!J7:J13)</f>
+        <v>0</v>
+      </c>
+      <c r="H19" s="18" t="n">
+        <f aca="false">SUM('World Cup 2026'!K7:K13)</f>
+        <v>0</v>
+      </c>
+      <c r="I19" s="19" t="n">
+        <f aca="false">I18+H19</f>
+        <v>4673.2</v>
+      </c>
+      <c r="J19" s="20" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="E20" s="24" t="n">
         <f aca="false">SUM('UFC 329'!F7:F15)</f>
         <v>1050</v>
       </c>
-      <c r="F16" s="16" t="n">
+      <c r="F20" s="24" t="n">
         <f aca="false">SUMIF('UFC 329'!I7:I15,"Pending",'UFC 329'!F7:F15)</f>
         <v>0</v>
       </c>
-      <c r="G16" s="17" t="n">
+      <c r="G20" s="25" t="n">
         <f aca="false">SUM('UFC 329'!J7:J15)</f>
         <v>1215.1103728313</v>
       </c>
-      <c r="H16" s="18" t="n">
+      <c r="H20" s="26" t="n">
         <f aca="false">SUM('UFC 329'!K7:K15)</f>
         <v>165.110372831303</v>
-      </c>
-      <c r="I16" s="19" t="n">
-        <f aca="false">B5+H16</f>
-        <v>5165.1103728313</v>
-      </c>
-      <c r="J16" s="20" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="n">
-        <v>2</v>
-      </c>
-      <c r="B17" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="C17" s="21" t="s">
-        <v>27</v>
-      </c>
-      <c r="D17" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="E17" s="24" t="n">
-        <f aca="false">SUM('World Cup 2026'!F7:F13)</f>
-        <v>1000</v>
-      </c>
-      <c r="F17" s="24" t="n">
-        <f aca="false">SUMIF('World Cup 2026'!I7:I13,"Pending",'World Cup 2026'!F7:F13)</f>
-        <v>1000</v>
-      </c>
-      <c r="G17" s="25" t="n">
-        <f aca="false">SUM('World Cup 2026'!J7:J13)</f>
-        <v>0</v>
-      </c>
-      <c r="H17" s="26" t="n">
-        <f aca="false">SUM('World Cup 2026'!K7:K13)</f>
-        <v>0</v>
-      </c>
-      <c r="I17" s="27" t="n">
-        <f aca="false">I16+H17</f>
-        <v>5165.1103728313</v>
-      </c>
-      <c r="J17" s="28" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="B18" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="C18" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="D18" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="E18" s="24" t="n">
-        <f aca="false">SUM('MLB Jul 12'!F7:F14)</f>
-        <v>1000</v>
-      </c>
-      <c r="F18" s="24" t="n">
-        <f aca="false">SUMIF('MLB Jul 12'!I7:I14,"Pending",'MLB Jul 12'!F7:F14)</f>
-        <v>200</v>
-      </c>
-      <c r="G18" s="25" t="n">
-        <f aca="false">SUM('MLB Jul 12'!J7:J14)</f>
-        <v>473.2</v>
-      </c>
-      <c r="H18" s="26" t="n">
-        <f aca="false">SUM('MLB Jul 12'!K7:K14)</f>
-        <v>-326.8</v>
-      </c>
-      <c r="I18" s="27" t="n">
-        <f aca="false">I17+H18</f>
-        <v>4838.3103728313</v>
-      </c>
-      <c r="J18" s="28" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="B19" s="22" t="s">
-        <v>33</v>
-      </c>
-      <c r="C19" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="D19" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="E19" s="24" t="n">
-        <f aca="false">SUM('NASCAR Jul 12'!F7:F13)</f>
-        <v>1000</v>
-      </c>
-      <c r="F19" s="24" t="n">
-        <f aca="false">SUMIF('NASCAR Jul 12'!I7:I13,"Pending",'NASCAR Jul 12'!F7:F13)</f>
-        <v>1000</v>
-      </c>
-      <c r="G19" s="25" t="n">
-        <f aca="false">SUM('NASCAR Jul 12'!J7:J13)</f>
-        <v>0</v>
-      </c>
-      <c r="H19" s="26" t="n">
-        <f aca="false">SUM('NASCAR Jul 12'!K7:K13)</f>
-        <v>0</v>
-      </c>
-      <c r="I19" s="27" t="n">
-        <f aca="false">I18+H19</f>
-        <v>4838.3103728313</v>
-      </c>
-      <c r="J19" s="28" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="n">
-        <v>5</v>
-      </c>
-      <c r="B20" s="22" t="s">
-        <v>35</v>
-      </c>
-      <c r="C20" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="D20" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="E20" s="24" t="n">
-        <f aca="false">SUM('WNBA Jul 12'!F7:F13)</f>
-        <v>1000</v>
-      </c>
-      <c r="F20" s="24" t="n">
-        <f aca="false">SUMIF('WNBA Jul 12'!I7:I13,"Pending",'WNBA Jul 12'!F7:F13)</f>
-        <v>1000</v>
-      </c>
-      <c r="G20" s="25" t="n">
-        <f aca="false">SUM('WNBA Jul 12'!J7:J13)</f>
-        <v>0</v>
-      </c>
-      <c r="H20" s="26" t="n">
-        <f aca="false">SUM('WNBA Jul 12'!K7:K13)</f>
-        <v>0</v>
       </c>
       <c r="I20" s="27" t="n">
         <f aca="false">I19+H20</f>

</xml_diff>

<commit_message>
MLB card settled: 3-5, -$197.77 (Giants ML won); balance $4,967.34
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011kwt7TrQj5DyWSPAGHQ9fr
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -100,15 +100,18 @@
     <t xml:space="preserve">2026-07-12</t>
   </si>
   <si>
+    <t xml:space="preserve">SETTLED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tab: MLB Jul 12 · SETTLED 3-5 (37.5%), -$197.77 · Giants ML won</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WNBA Sunday Doubleheader</t>
+  </si>
+  <si>
     <t xml:space="preserve">ACTIVE</t>
   </si>
   <si>
-    <t xml:space="preserve">Tab: MLB Jul 12 · LIVE — 2-5 thru 7, Giants ML remaining</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WNBA Sunday Doubleheader</t>
-  </si>
-  <si>
     <t xml:space="preserve">Tab: WNBA Jul 12 · Sky@Wings 7 ET, Fever@Aces 9 ET</t>
   </si>
   <si>
@@ -133,9 +136,6 @@
     <t xml:space="preserve">2026-07-11</t>
   </si>
   <si>
-    <t xml:space="preserve">SETTLED</t>
-  </si>
-  <si>
     <t xml:space="preserve">Tab: UFC 329 · 6-3, settled Jul 11 · archives Jul 18</t>
   </si>
   <si>
@@ -643,7 +643,7 @@
     <t xml:space="preserve">TEST 3 — MLB SUNDAY SLATE · JULY 12, 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">STATUS: ACTIVE — 1 of 8 settled (Pirates ✓ +$135.20)</t>
+    <t xml:space="preserve">STATUS: ARCHIVED — settled Jul 12 (3-5, -$197.77)</t>
   </si>
   <si>
     <t xml:space="preserve">15-game slate, 8 bets · Source: mlb-jul12-betting-card.html · Lines: ESPN consensus board, Sunday AM · Research: VSiN, PickDawgz, DK Network</t>
@@ -664,7 +664,7 @@
     <t xml:space="preserve">vs Rockies · McDonald vs Lorenzen (6.46 ERA)</t>
   </si>
   <si>
-    <t xml:space="preserve">Safest play — Lorenzen 1.4 HR/9, Rockies worst road team</t>
+    <t xml:space="preserve">Safest play — Lorenzen 1.4 HR/9, Rockies worst road team · RESULT: SF 3-1 · Lorenzen fade lands</t>
   </si>
   <si>
     <t xml:space="preserve">Athletics ML</t>
@@ -1160,20 +1160,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="13">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
     <numFmt numFmtId="167" formatCode="\$#,##0.00"/>
-    <numFmt numFmtId="168" formatCode="\$#,##0"/>
-    <numFmt numFmtId="169" formatCode="\$#,##0.00"/>
-    <numFmt numFmtId="170" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
-    <numFmt numFmtId="171" formatCode="\+0;\-0"/>
-    <numFmt numFmtId="172" formatCode="0"/>
-    <numFmt numFmtId="173" formatCode="0.0%"/>
-    <numFmt numFmtId="174" formatCode="0%"/>
-    <numFmt numFmtId="175" formatCode="0.0&quot; exp. wins&quot;"/>
-    <numFmt numFmtId="176" formatCode="0.0"/>
+    <numFmt numFmtId="168" formatCode="\+0;\-0"/>
+    <numFmt numFmtId="169" formatCode="0"/>
+    <numFmt numFmtId="170" formatCode="0.0%"/>
+    <numFmt numFmtId="171" formatCode="0%"/>
+    <numFmt numFmtId="172" formatCode="0.0&quot; exp. wins&quot;"/>
+    <numFmt numFmtId="173" formatCode="0.0"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -1254,7 +1251,7 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <color rgb="FF1B7A3D"/>
+      <color rgb="FF808080"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1269,7 +1266,7 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <color rgb="FF808080"/>
+      <color rgb="FF1B7A3D"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1363,14 +1360,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE2F0D9"/>
-        <bgColor rgb="FFE7E6E6"/>
+        <fgColor rgb="FFE7E6E6"/>
+        <bgColor rgb="FFE2F0D9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE7E6E6"/>
-        <bgColor rgb="FFE2F0D9"/>
+        <fgColor rgb="FFE2F0D9"/>
+        <bgColor rgb="FFE7E6E6"/>
       </patternFill>
     </fill>
     <fill>
@@ -1530,19 +1527,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1562,19 +1559,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1642,39 +1639,67 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="168" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="171" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="172" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1682,34 +1707,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="174" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="175" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="176" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1722,7 +1719,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1738,7 +1735,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2071,7 +2068,7 @@
       </c>
       <c r="B6" s="7" t="n">
         <f aca="false">H21</f>
-        <v>-161.689627168697</v>
+        <v>-32.6573691041808</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2080,7 +2077,7 @@
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">I20</f>
-        <v>4838.3103728313</v>
+        <v>4967.34263089582</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2089,7 +2086,7 @@
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">F21</f>
-        <v>3200</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2098,7 +2095,7 @@
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">B7-B8</f>
-        <v>1638.3103728313</v>
+        <v>1967.34263089582</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2107,7 +2104,7 @@
       </c>
       <c r="B10" s="10" t="str">
         <f aca="false">COUNTIF(D16:D20,"ACTIVE")&amp;" of 4 max"</f>
-        <v>4 of 4 max</v>
+        <v>3 of 4 max</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2174,169 +2171,169 @@
       </c>
       <c r="F16" s="16" t="n">
         <f aca="false">SUMIF('MLB Jul 12'!I7:I14,"Pending",'MLB Jul 12'!F7:F14)</f>
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="G16" s="17" t="n">
         <f aca="false">SUM('MLB Jul 12'!J7:J14)</f>
-        <v>473.2</v>
+        <v>802.232258064516</v>
       </c>
       <c r="H16" s="18" t="n">
         <f aca="false">SUM('MLB Jul 12'!K7:K14)</f>
-        <v>-326.8</v>
+        <v>-197.767741935484</v>
       </c>
       <c r="I16" s="19" t="n">
         <f aca="false">B5+H16</f>
-        <v>4673.2</v>
+        <v>4802.23225806452</v>
       </c>
       <c r="J16" s="20" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="n">
+      <c r="A17" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="B17" s="14" t="s">
+      <c r="B17" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="C17" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="D17" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="E17" s="16" t="n">
+      <c r="D17" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17" s="24" t="n">
         <f aca="false">SUM('WNBA Jul 12'!F7:F13)</f>
         <v>1000</v>
       </c>
-      <c r="F17" s="16" t="n">
+      <c r="F17" s="24" t="n">
         <f aca="false">SUMIF('WNBA Jul 12'!I7:I13,"Pending",'WNBA Jul 12'!F7:F13)</f>
         <v>1000</v>
       </c>
-      <c r="G17" s="17" t="n">
+      <c r="G17" s="25" t="n">
         <f aca="false">SUM('WNBA Jul 12'!J7:J13)</f>
         <v>0</v>
       </c>
-      <c r="H17" s="18" t="n">
+      <c r="H17" s="26" t="n">
         <f aca="false">SUM('WNBA Jul 12'!K7:K13)</f>
         <v>0</v>
       </c>
-      <c r="I17" s="19" t="n">
+      <c r="I17" s="27" t="n">
         <f aca="false">I16+H17</f>
-        <v>4673.2</v>
-      </c>
-      <c r="J17" s="20" t="s">
+        <v>4802.23225806452</v>
+      </c>
+      <c r="J17" s="28" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" s="23" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="C18" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="D18" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="E18" s="16" t="n">
+      <c r="E18" s="24" t="n">
         <f aca="false">SUM('NASCAR Jul 12'!F7:F13)</f>
         <v>1000</v>
       </c>
-      <c r="F18" s="16" t="n">
+      <c r="F18" s="24" t="n">
         <f aca="false">SUMIF('NASCAR Jul 12'!I7:I13,"Pending",'NASCAR Jul 12'!F7:F13)</f>
         <v>1000</v>
       </c>
-      <c r="G18" s="17" t="n">
+      <c r="G18" s="25" t="n">
         <f aca="false">SUM('NASCAR Jul 12'!J7:J13)</f>
         <v>0</v>
       </c>
-      <c r="H18" s="18" t="n">
+      <c r="H18" s="26" t="n">
         <f aca="false">SUM('NASCAR Jul 12'!K7:K13)</f>
         <v>0</v>
       </c>
-      <c r="I18" s="19" t="n">
+      <c r="I18" s="27" t="n">
         <f aca="false">I17+H18</f>
-        <v>4673.2</v>
-      </c>
-      <c r="J18" s="20" t="s">
-        <v>29</v>
+        <v>4802.23225806452</v>
+      </c>
+      <c r="J18" s="28" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="n">
+      <c r="A19" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="B19" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="C19" s="13" t="s">
+      <c r="B19" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="D19" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="E19" s="16" t="n">
+      <c r="C19" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" s="24" t="n">
         <f aca="false">SUM('World Cup 2026'!F7:F13)</f>
         <v>1000</v>
       </c>
-      <c r="F19" s="16" t="n">
+      <c r="F19" s="24" t="n">
         <f aca="false">SUMIF('World Cup 2026'!I7:I13,"Pending",'World Cup 2026'!F7:F13)</f>
         <v>1000</v>
       </c>
-      <c r="G19" s="17" t="n">
+      <c r="G19" s="25" t="n">
         <f aca="false">SUM('World Cup 2026'!J7:J13)</f>
         <v>0</v>
       </c>
-      <c r="H19" s="18" t="n">
+      <c r="H19" s="26" t="n">
         <f aca="false">SUM('World Cup 2026'!K7:K13)</f>
         <v>0</v>
       </c>
-      <c r="I19" s="19" t="n">
+      <c r="I19" s="27" t="n">
         <f aca="false">I18+H19</f>
-        <v>4673.2</v>
-      </c>
-      <c r="J19" s="20" t="s">
-        <v>32</v>
+        <v>4802.23225806452</v>
+      </c>
+      <c r="J19" s="28" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="n">
+      <c r="A20" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="B20" s="22" t="s">
-        <v>33</v>
-      </c>
-      <c r="C20" s="21" t="s">
+      <c r="B20" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="D20" s="23" t="s">
+      <c r="C20" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="E20" s="24" t="n">
+      <c r="D20" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E20" s="16" t="n">
         <f aca="false">SUM('UFC 329'!F7:F15)</f>
         <v>1050</v>
       </c>
-      <c r="F20" s="24" t="n">
+      <c r="F20" s="16" t="n">
         <f aca="false">SUMIF('UFC 329'!I7:I15,"Pending",'UFC 329'!F7:F15)</f>
         <v>0</v>
       </c>
-      <c r="G20" s="25" t="n">
+      <c r="G20" s="17" t="n">
         <f aca="false">SUM('UFC 329'!J7:J15)</f>
         <v>1215.1103728313</v>
       </c>
-      <c r="H20" s="26" t="n">
+      <c r="H20" s="18" t="n">
         <f aca="false">SUM('UFC 329'!K7:K15)</f>
         <v>165.110372831303</v>
       </c>
-      <c r="I20" s="27" t="n">
+      <c r="I20" s="19" t="n">
         <f aca="false">I19+H20</f>
-        <v>4838.3103728313</v>
-      </c>
-      <c r="J20" s="28" t="s">
+        <v>4967.34263089582</v>
+      </c>
+      <c r="J20" s="20" t="s">
         <v>36</v>
       </c>
     </row>
@@ -2353,15 +2350,15 @@
       </c>
       <c r="F21" s="31" t="n">
         <f aca="false">SUM(F16:F20)</f>
-        <v>3200</v>
+        <v>3000</v>
       </c>
       <c r="G21" s="32" t="n">
         <f aca="false">SUM(G16:G20)</f>
-        <v>1688.3103728313</v>
+        <v>2017.34263089582</v>
       </c>
       <c r="H21" s="33" t="n">
         <f aca="false">SUM(H16:H20)</f>
-        <v>-161.689627168697</v>
+        <v>-32.6573691041808</v>
       </c>
       <c r="I21" s="29"/>
       <c r="J21" s="29"/>
@@ -3944,7 +3941,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF1B7A3D"/>
+    <tabColor rgb="FF808080"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M42"/>
@@ -3966,7 +3963,7 @@
       <c r="A1" s="39" t="s">
         <v>204</v>
       </c>
-      <c r="H1" s="56" t="s">
+      <c r="H1" s="40" t="s">
         <v>205</v>
       </c>
     </row>
@@ -4053,16 +4050,16 @@
         <f aca="false">F7+G7</f>
         <v>329.032258064516</v>
       </c>
-      <c r="I7" s="57" t="s">
-        <v>112</v>
+      <c r="I7" s="46" t="s">
+        <v>79</v>
       </c>
       <c r="J7" s="45" t="n">
         <f aca="false">IF(I7="Win",F7+G7,IF(I7="Push",F7,IF(I7="Loss",0,0)))</f>
-        <v>0</v>
+        <v>329.032258064516</v>
       </c>
       <c r="K7" s="47" t="n">
         <f aca="false">IF(I7="Pending",0,J7-F7)</f>
-        <v>0</v>
+        <v>129.032258064516</v>
       </c>
       <c r="L7" s="58" t="n">
         <v>0.62</v>
@@ -4409,11 +4406,11 @@
       <c r="I15" s="50"/>
       <c r="J15" s="32" t="n">
         <f aca="false">SUM(J7:J14)</f>
-        <v>473.2</v>
+        <v>802.232258064516</v>
       </c>
       <c r="K15" s="33" t="n">
         <f aca="false">SUM(K7:K14)</f>
-        <v>-326.8</v>
+        <v>-197.767741935484</v>
       </c>
       <c r="L15" s="59" t="n">
         <f aca="false">SUM(L7:L14)</f>
@@ -4432,7 +4429,7 @@
       </c>
       <c r="C18" s="52" t="n">
         <f aca="false">COUNTIF(I7:I14,"Win")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4459,7 +4456,7 @@
       </c>
       <c r="C21" s="52" t="n">
         <f aca="false">COUNTIF(I7:I14,"Pending")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4468,7 +4465,7 @@
       </c>
       <c r="C22" s="53" t="n">
         <f aca="false">IF(COUNTIF(I7:I14,"Win")+COUNTIF(I7:I14,"Loss")=0,"—",COUNTIF(I7:I14,"Win")/(COUNTIF(I7:I14,"Win")+COUNTIF(I7:I14,"Loss")))</f>
-        <v>0.285714285714286</v>
+        <v>0.375</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4486,7 +4483,7 @@
       </c>
       <c r="C24" s="45" t="n">
         <f aca="false">SUM(J7:J14)</f>
-        <v>473.2</v>
+        <v>802.232258064516</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4495,7 +4492,7 @@
       </c>
       <c r="C25" s="47" t="n">
         <f aca="false">SUM(K7:K14)</f>
-        <v>-326.8</v>
+        <v>-197.767741935484</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4504,7 +4501,7 @@
       </c>
       <c r="C26" s="53" t="n">
         <f aca="false">IF(SUM(F7:F14)=0,"—",SUM(K7:K14)/SUM(F7:F14))</f>
-        <v>-0.3268</v>
+        <v>-0.197767741935484</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Aces -4.5 covers on comeback (+$138.89); WNBA 2-3, props pending box score
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011kwt7TrQj5DyWSPAGHQ9fr
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -104,7 +104,7 @@
     <t xml:space="preserve">ACTIVE</t>
   </si>
   <si>
-    <t xml:space="preserve">Tab: WNBA Jul 12 · Game 1: 1-3 incl. parlay (-$355.66) · Aces game live</t>
+    <t xml:space="preserve">Tab: WNBA Jul 12 · 2-3, Wilson DD &amp; Mitchell 3s pending box score</t>
   </si>
   <si>
     <t xml:space="preserve">NASCAR Quaker State 400</t>
@@ -1193,7 +1193,7 @@
     <t xml:space="preserve">vs Fever · 9 PM ET</t>
   </si>
   <si>
-    <t xml:space="preserve">+41 differential last 7 home w/ Wilson; rested off 48-pt blowout Sat</t>
+    <t xml:space="preserve">+41 differential last 7 home w/ Wilson; rested off 48-pt blowout Sat · RESULT: Aces won by 6-8 (CBS final 115/117-109) after huge 4th-qtr rally — covered</t>
   </si>
   <si>
     <t xml:space="preserve">A'ja Wilson Double-Double (Yes)</t>
@@ -2253,7 +2253,7 @@
       </c>
       <c r="B6" s="7" t="n">
         <f aca="false">H23</f>
-        <v>-388.317746462671</v>
+        <v>-249.428857573782</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2262,7 +2262,7 @@
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">B5+B6</f>
-        <v>4611.68225353733</v>
+        <v>4750.57114242622</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">F23</f>
-        <v>3000</v>
+        <v>2850</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2280,7 +2280,7 @@
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">B7-B8</f>
-        <v>1611.68225353733</v>
+        <v>1900.57114242622</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2356,19 +2356,19 @@
       </c>
       <c r="F16" s="16" t="n">
         <f aca="false">SUMIF('WNBA Jul 12'!I7:I13,"Pending",'WNBA Jul 12'!F7:F13)</f>
-        <v>400</v>
+        <v>250</v>
       </c>
       <c r="G16" s="17" t="n">
         <f aca="false">SUM('WNBA Jul 12'!J7:J13)</f>
-        <v>244.339622641509</v>
+        <v>533.228511530398</v>
       </c>
       <c r="H16" s="18" t="n">
         <f aca="false">SUM('WNBA Jul 12'!K7:K13)</f>
-        <v>-355.660377358491</v>
+        <v>-216.771488469602</v>
       </c>
       <c r="I16" s="19" t="n">
         <f aca="false">B5+H16</f>
-        <v>4644.33962264151</v>
+        <v>4783.2285115304</v>
       </c>
       <c r="J16" s="20" t="s">
         <v>25</v>
@@ -2405,7 +2405,7 @@
       </c>
       <c r="I17" s="19" t="n">
         <f aca="false">I16+H17</f>
-        <v>4644.33962264151</v>
+        <v>4783.2285115304</v>
       </c>
       <c r="J17" s="20" t="s">
         <v>27</v>
@@ -2442,7 +2442,7 @@
       </c>
       <c r="I18" s="19" t="n">
         <f aca="false">I17+H18</f>
-        <v>4644.33962264151</v>
+        <v>4783.2285115304</v>
       </c>
       <c r="J18" s="20" t="s">
         <v>30</v>
@@ -2479,7 +2479,7 @@
       </c>
       <c r="I19" s="19" t="n">
         <f aca="false">I18+H19</f>
-        <v>4644.33962264151</v>
+        <v>4783.2285115304</v>
       </c>
       <c r="J19" s="20" t="s">
         <v>33</v>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="I20" s="27" t="n">
         <f aca="false">I19+H20</f>
-        <v>4644.33962264151</v>
+        <v>4783.2285115304</v>
       </c>
       <c r="J20" s="28" t="s">
         <v>37</v>
@@ -2549,7 +2549,7 @@
       </c>
       <c r="I21" s="35" t="n">
         <f aca="false">I20+H21</f>
-        <v>4446.57188070603</v>
+        <v>4585.46076959491</v>
       </c>
       <c r="J21" s="36" t="s">
         <v>40</v>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="I22" s="35" t="n">
         <f aca="false">I21+H22</f>
-        <v>4611.68225353733</v>
+        <v>4750.57114242622</v>
       </c>
       <c r="J22" s="36" t="s">
         <v>43</v>
@@ -2605,15 +2605,15 @@
       </c>
       <c r="F23" s="39" t="n">
         <f aca="false">SUM(F16:F22)</f>
-        <v>3000</v>
+        <v>2850</v>
       </c>
       <c r="G23" s="40" t="n">
         <f aca="false">SUM(G16:G22)</f>
-        <v>2261.68225353733</v>
+        <v>2550.57114242622</v>
       </c>
       <c r="H23" s="41" t="n">
         <f aca="false">SUM(H16:H22)</f>
-        <v>-388.317746462671</v>
+        <v>-249.428857573782</v>
       </c>
       <c r="I23" s="37"/>
       <c r="J23" s="37"/>
@@ -6239,16 +6239,16 @@
         <f aca="false">F10+G10</f>
         <v>288.888888888889</v>
       </c>
-      <c r="I10" s="65" t="s">
-        <v>126</v>
+      <c r="I10" s="54" t="s">
+        <v>93</v>
       </c>
       <c r="J10" s="53" t="n">
         <f aca="false">IF(I10="Win",F10+G10,IF(I10="Push",F10,IF(I10="Loss",0,0)))</f>
-        <v>0</v>
+        <v>288.888888888889</v>
       </c>
       <c r="K10" s="55" t="n">
         <f aca="false">IF(I10="Pending",0,J10-F10)</f>
-        <v>0</v>
+        <v>138.888888888889</v>
       </c>
       <c r="L10" s="66" t="n">
         <v>0.55</v>
@@ -6415,11 +6415,11 @@
       <c r="I14" s="37"/>
       <c r="J14" s="40" t="n">
         <f aca="false">SUM(J7:J13)</f>
-        <v>244.339622641509</v>
+        <v>533.228511530398</v>
       </c>
       <c r="K14" s="41" t="n">
         <f aca="false">SUM(K7:K13)</f>
-        <v>-355.660377358491</v>
+        <v>-216.771488469602</v>
       </c>
       <c r="L14" s="67" t="n">
         <f aca="false">SUM(L7:L13)</f>
@@ -6438,7 +6438,7 @@
       </c>
       <c r="C17" s="60" t="n">
         <f aca="false">COUNTIF(I7:I13,"Win")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6465,7 +6465,7 @@
       </c>
       <c r="C20" s="60" t="n">
         <f aca="false">COUNTIF(I7:I13,"Pending")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6474,7 +6474,7 @@
       </c>
       <c r="C21" s="61" t="n">
         <f aca="false">IF(COUNTIF(I7:I13,"Win")+COUNTIF(I7:I13,"Loss")=0,"—",COUNTIF(I7:I13,"Win")/(COUNTIF(I7:I13,"Win")+COUNTIF(I7:I13,"Loss")))</f>
-        <v>0.25</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6492,7 +6492,7 @@
       </c>
       <c r="C23" s="53" t="n">
         <f aca="false">SUM(J7:J13)</f>
-        <v>244.339622641509</v>
+        <v>533.228511530398</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6501,7 +6501,7 @@
       </c>
       <c r="C24" s="55" t="n">
         <f aca="false">SUM(K7:K13)</f>
-        <v>-355.660377358491</v>
+        <v>-216.771488469602</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6510,7 +6510,7 @@
       </c>
       <c r="C25" s="61" t="n">
         <f aca="false">IF(SUM(F7:F13)=0,"—",SUM(K7:K13)/SUM(F7:F13))</f>
-        <v>-0.355660377358491</v>
+        <v>-0.216771488469602</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
WNBA Jul 12 card settled: 3-4, -$298.15 (Fever routed Aces 109-75; Wilson DD 20/12 + Mitchell 3 threes cash, Aces -4.5 dead); corrects interim commit 5116958 which graded Aces -4.5 as a cover before the final (verified: ESPN + TSN); NASCAR red-flag status; balance $4,669.19
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QcpfLBxkPb1dDWHh7szCcL
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -95,60 +95,60 @@
     <t xml:space="preserve">Detail Tab / Notes</t>
   </si>
   <si>
+    <t xml:space="preserve">NASCAR Quaker State 400</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACTIVE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tab: NASCAR Jul 12 · red-flag lightning delay at lap 109 · finish ~1 AM CT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">World Cup 2026 — Final Four</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jul 14-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tab: World Cup 2026 · semis Tue/Wed, final Sun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Open Championship (golf)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jul 16-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tab: The Open · $600 outrights + $400 props Wed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rugby Nations Cup — Final Rd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUEUED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Draft card built · odds post ~Fri · $0 at risk</t>
+  </si>
+  <si>
     <t xml:space="preserve">WNBA Sunday Doubleheader</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-07-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ACTIVE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tab: WNBA Jul 12 · 2-3, Wilson DD &amp; Mitchell 3s pending box score</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NASCAR Quaker State 400</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tab: NASCAR Jul 12 · race ~7 PM ET tonight</t>
-  </si>
-  <si>
-    <t xml:space="preserve">World Cup 2026 — Final Four</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jul 14-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tab: World Cup 2026 · semis Tue/Wed, final Sun</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Open Championship (golf)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jul 16-19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tab: The Open · $600 outrights + $400 props Wed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rugby Nations Cup — Final Rd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-07-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QUEUED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Draft card built · odds post ~Fri · $0 at risk</t>
+    <t xml:space="preserve">SETTLED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tab: WNBA Jul 12 · SETTLED 3-4 (42.9%), -$298.15 · Fever routed Aces 109-75</t>
   </si>
   <si>
     <t xml:space="preserve">MLB Sunday Slate (15 games)</t>
   </si>
   <si>
-    <t xml:space="preserve">SETTLED</t>
-  </si>
-  <si>
     <t xml:space="preserve">Tab: MLB Jul 12 · SETTLED 3-5 (37.5%), -$197.77</t>
   </si>
   <si>
@@ -866,7 +866,7 @@
     <t xml:space="preserve">TEST 4 — NASCAR QUAKER STATE 400 · ECHOPARK SPEEDWAY (ATLANTA) · JULY 12, 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">STATUS: ACTIVE — race ~7 PM ET tonight</t>
+    <t xml:space="preserve">STATUS: ACTIVE — red-flagged (lightning) at lap 109/260; finish expected ~1 AM CT</t>
   </si>
   <si>
     <t xml:space="preserve">Race ~7:00 PM ET on TNT · Source: nascar-jul12-betting-card.html · Odds: Covers/VSiN/CBS (FanDuel) consensus, Sunday PM</t>
@@ -1148,7 +1148,7 @@
     <t xml:space="preserve">TEST 5 — WNBA SUNDAY NIGHT DOUBLEHEADER · JULY 12, 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">STATUS: ACTIVE — Game 1 graded 1-2; Fever@Aces in progress</t>
+    <t xml:space="preserve">STATUS: SETTLED — 3-4 (42.9%), -$298.15 · Fever routed Aces 109-75</t>
   </si>
   <si>
     <t xml:space="preserve">Sky @ Wings 7 PM ET (ESPN) · Fever @ Aces 9 PM ET (NBC) · Source: wnba-jul12-betting-card.html · Lines: FanDuel via SI Betting / Covers, ~5 PM CT</t>
@@ -1193,7 +1193,7 @@
     <t xml:space="preserve">vs Fever · 9 PM ET</t>
   </si>
   <si>
-    <t xml:space="preserve">+41 differential last 7 home w/ Wilson; rested off 48-pt blowout Sat · RESULT: Aces won by 6-8 (CBS final 115/117-109) after huge 4th-qtr rally — covered</t>
+    <t xml:space="preserve">+41 differential last 7 home w/ Wilson; rested off 48-pt blowout Sat · RESULT: Fever 109-75 — Aces lost by 34, spread dead</t>
   </si>
   <si>
     <t xml:space="preserve">A'ja Wilson Double-Double (Yes)</t>
@@ -1202,7 +1202,7 @@
     <t xml:space="preserve">Aces F · player prop</t>
   </si>
   <si>
-    <t xml:space="preserve">DD in 5 straight career games vs Clark; 10.8 reb/game at home; 11 DDs (3rd in W)</t>
+    <t xml:space="preserve">DD in 5 straight career games vs Clark; 10.8 reb/game at home; 11 DDs (3rd in W) · RESULT: Wilson 20 pts / 12 reb — double-double cashed</t>
   </si>
   <si>
     <t xml:space="preserve">Kelsey Mitchell Over 2.5 Threes</t>
@@ -1211,7 +1211,7 @@
     <t xml:space="preserve">Fever G · player prop</t>
   </si>
   <si>
-    <t xml:space="preserve">3+ threes in 6 straight, 8 of 10; 41.1% from deep; LV 12th vs opp threes</t>
+    <t xml:space="preserve">3+ threes in 6 straight, 8 of 10; 41.1% from deep; LV 12th vs opp threes · RESULT: Mitchell 3-of-8 from deep (27 pts) — cleared 2.5</t>
   </si>
   <si>
     <t xml:space="preserve">LONGSHOT: 4-Leg Parlay</t>
@@ -2253,7 +2253,7 @@
       </c>
       <c r="B6" s="7" t="n">
         <f aca="false">H23</f>
-        <v>-249.428857573782</v>
+        <v>-330.81085941033</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2262,7 +2262,7 @@
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">B5+B6</f>
-        <v>4750.57114242622</v>
+        <v>4669.18914058967</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">F23</f>
-        <v>2850</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2280,7 +2280,7 @@
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">B7-B8</f>
-        <v>1900.57114242622</v>
+        <v>2069.18914058967</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="B10" s="10" t="str">
         <f aca="false">COUNTIF(D16:D22,"ACTIVE")&amp;" of 4 max"</f>
-        <v>4 of 4 max</v>
+        <v>3 of 4 max</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2339,7 +2339,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B16" s="14" t="s">
         <v>22</v>
@@ -2351,171 +2351,171 @@
         <v>24</v>
       </c>
       <c r="E16" s="16" t="n">
+        <f aca="false">SUM('NASCAR Jul 12'!F7:F13)</f>
+        <v>1000</v>
+      </c>
+      <c r="F16" s="16" t="n">
+        <f aca="false">SUMIF('NASCAR Jul 12'!I7:I13,"Pending",'NASCAR Jul 12'!F7:F13)</f>
+        <v>1000</v>
+      </c>
+      <c r="G16" s="17" t="n">
+        <f aca="false">SUM('NASCAR Jul 12'!J7:J13)</f>
+        <v>0</v>
+      </c>
+      <c r="H16" s="18" t="n">
+        <f aca="false">SUM('NASCAR Jul 12'!K7:K13)</f>
+        <v>0</v>
+      </c>
+      <c r="I16" s="19" t="n">
+        <f aca="false">B5+H16</f>
+        <v>5000</v>
+      </c>
+      <c r="J16" s="20" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E17" s="16" t="n">
+        <f aca="false">SUM('World Cup 2026'!F7:F13)</f>
+        <v>1000</v>
+      </c>
+      <c r="F17" s="16" t="n">
+        <f aca="false">SUMIF('World Cup 2026'!I7:I13,"Pending",'World Cup 2026'!F7:F13)</f>
+        <v>1000</v>
+      </c>
+      <c r="G17" s="17" t="n">
+        <f aca="false">SUM('World Cup 2026'!J7:J13)</f>
+        <v>0</v>
+      </c>
+      <c r="H17" s="18" t="n">
+        <f aca="false">SUM('World Cup 2026'!K7:K13)</f>
+        <v>0</v>
+      </c>
+      <c r="I17" s="19" t="n">
+        <f aca="false">I16+H17</f>
+        <v>5000</v>
+      </c>
+      <c r="J17" s="20" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D18" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E18" s="16" t="n">
+        <f aca="false">SUM('The Open'!F7:F12)</f>
+        <v>600</v>
+      </c>
+      <c r="F18" s="16" t="n">
+        <f aca="false">SUMIF('The Open'!I7:I12,"Pending",'The Open'!F7:F12)</f>
+        <v>600</v>
+      </c>
+      <c r="G18" s="17" t="n">
+        <f aca="false">SUM('The Open'!J7:J12)</f>
+        <v>0</v>
+      </c>
+      <c r="H18" s="18" t="n">
+        <f aca="false">SUM('The Open'!K7:K12)</f>
+        <v>0</v>
+      </c>
+      <c r="I18" s="19" t="n">
+        <f aca="false">I17+H18</f>
+        <v>5000</v>
+      </c>
+      <c r="J18" s="20" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="21" t="n">
+        <v>7</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="E19" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="27" t="n">
+        <f aca="false">I18+H19</f>
+        <v>5000</v>
+      </c>
+      <c r="J19" s="28" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="B20" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="C20" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="D20" s="31" t="s">
+        <v>37</v>
+      </c>
+      <c r="E20" s="32" t="n">
         <f aca="false">SUM('WNBA Jul 12'!F7:F13)</f>
         <v>1000</v>
       </c>
-      <c r="F16" s="16" t="n">
+      <c r="F20" s="32" t="n">
         <f aca="false">SUMIF('WNBA Jul 12'!I7:I13,"Pending",'WNBA Jul 12'!F7:F13)</f>
-        <v>250</v>
-      </c>
-      <c r="G16" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="33" t="n">
         <f aca="false">SUM('WNBA Jul 12'!J7:J13)</f>
-        <v>533.228511530398</v>
-      </c>
-      <c r="H16" s="18" t="n">
+        <v>701.846509693851</v>
+      </c>
+      <c r="H20" s="34" t="n">
         <f aca="false">SUM('WNBA Jul 12'!K7:K13)</f>
-        <v>-216.771488469602</v>
-      </c>
-      <c r="I16" s="19" t="n">
-        <f aca="false">B5+H16</f>
-        <v>4783.2285115304</v>
-      </c>
-      <c r="J16" s="20" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="B17" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="D17" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="E17" s="16" t="n">
-        <f aca="false">SUM('NASCAR Jul 12'!F7:F13)</f>
-        <v>1000</v>
-      </c>
-      <c r="F17" s="16" t="n">
-        <f aca="false">SUMIF('NASCAR Jul 12'!I7:I13,"Pending",'NASCAR Jul 12'!F7:F13)</f>
-        <v>1000</v>
-      </c>
-      <c r="G17" s="17" t="n">
-        <f aca="false">SUM('NASCAR Jul 12'!J7:J13)</f>
-        <v>0</v>
-      </c>
-      <c r="H17" s="18" t="n">
-        <f aca="false">SUM('NASCAR Jul 12'!K7:K13)</f>
-        <v>0</v>
-      </c>
-      <c r="I17" s="19" t="n">
-        <f aca="false">I16+H17</f>
-        <v>4783.2285115304</v>
-      </c>
-      <c r="J17" s="20" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="C18" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="D18" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="E18" s="16" t="n">
-        <f aca="false">SUM('World Cup 2026'!F7:F13)</f>
-        <v>1000</v>
-      </c>
-      <c r="F18" s="16" t="n">
-        <f aca="false">SUMIF('World Cup 2026'!I7:I13,"Pending",'World Cup 2026'!F7:F13)</f>
-        <v>1000</v>
-      </c>
-      <c r="G18" s="17" t="n">
-        <f aca="false">SUM('World Cup 2026'!J7:J13)</f>
-        <v>0</v>
-      </c>
-      <c r="H18" s="18" t="n">
-        <f aca="false">SUM('World Cup 2026'!K7:K13)</f>
-        <v>0</v>
-      </c>
-      <c r="I18" s="19" t="n">
-        <f aca="false">I17+H18</f>
-        <v>4783.2285115304</v>
-      </c>
-      <c r="J18" s="20" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="B19" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="C19" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="D19" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="E19" s="16" t="n">
-        <f aca="false">SUM('The Open'!F7:F12)</f>
-        <v>600</v>
-      </c>
-      <c r="F19" s="16" t="n">
-        <f aca="false">SUMIF('The Open'!I7:I12,"Pending",'The Open'!F7:F12)</f>
-        <v>600</v>
-      </c>
-      <c r="G19" s="17" t="n">
-        <f aca="false">SUM('The Open'!J7:J12)</f>
-        <v>0</v>
-      </c>
-      <c r="H19" s="18" t="n">
-        <f aca="false">SUM('The Open'!K7:K12)</f>
-        <v>0</v>
-      </c>
-      <c r="I19" s="19" t="n">
-        <f aca="false">I18+H19</f>
-        <v>4783.2285115304</v>
-      </c>
-      <c r="J19" s="20" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="n">
-        <v>7</v>
-      </c>
-      <c r="B20" s="22" t="s">
-        <v>34</v>
-      </c>
-      <c r="C20" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="D20" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="E20" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" s="27" t="n">
+        <v>-298.153490306149</v>
+      </c>
+      <c r="I20" s="35" t="n">
         <f aca="false">I19+H20</f>
-        <v>4783.2285115304</v>
-      </c>
-      <c r="J20" s="28" t="s">
-        <v>37</v>
+        <v>4701.84650969385</v>
+      </c>
+      <c r="J20" s="36" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2523,13 +2523,13 @@
         <v>3</v>
       </c>
       <c r="B21" s="30" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C21" s="29" t="s">
         <v>23</v>
       </c>
       <c r="D21" s="31" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E21" s="32" t="n">
         <f aca="false">SUM('MLB Jul 12'!F7:F14)</f>
@@ -2549,7 +2549,7 @@
       </c>
       <c r="I21" s="35" t="n">
         <f aca="false">I20+H21</f>
-        <v>4585.46076959491</v>
+        <v>4504.07876775837</v>
       </c>
       <c r="J21" s="36" t="s">
         <v>40</v>
@@ -2566,7 +2566,7 @@
         <v>42</v>
       </c>
       <c r="D22" s="31" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E22" s="32" t="n">
         <f aca="false">SUM('UFC 329'!F7:F15)</f>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="I22" s="35" t="n">
         <f aca="false">I21+H22</f>
-        <v>4750.57114242622</v>
+        <v>4669.18914058967</v>
       </c>
       <c r="J22" s="36" t="s">
         <v>43</v>
@@ -2605,15 +2605,15 @@
       </c>
       <c r="F23" s="39" t="n">
         <f aca="false">SUM(F16:F22)</f>
-        <v>2850</v>
+        <v>2600</v>
       </c>
       <c r="G23" s="40" t="n">
         <f aca="false">SUM(G16:G22)</f>
-        <v>2550.57114242622</v>
+        <v>2719.18914058967</v>
       </c>
       <c r="H23" s="41" t="n">
         <f aca="false">SUM(H16:H22)</f>
-        <v>-249.428857573782</v>
+        <v>-330.81085941033</v>
       </c>
       <c r="I23" s="37"/>
       <c r="J23" s="37"/>
@@ -5995,7 +5995,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF1B7A3D"/>
+    <tabColor rgb="FF808080"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M30"/>
@@ -6239,16 +6239,16 @@
         <f aca="false">F10+G10</f>
         <v>288.888888888889</v>
       </c>
-      <c r="I10" s="54" t="s">
-        <v>93</v>
+      <c r="I10" s="65" t="s">
+        <v>101</v>
       </c>
       <c r="J10" s="53" t="n">
         <f aca="false">IF(I10="Win",F10+G10,IF(I10="Push",F10,IF(I10="Loss",0,0)))</f>
-        <v>288.888888888889</v>
+        <v>0</v>
       </c>
       <c r="K10" s="55" t="n">
         <f aca="false">IF(I10="Pending",0,J10-F10)</f>
-        <v>138.888888888889</v>
+        <v>-150</v>
       </c>
       <c r="L10" s="66" t="n">
         <v>0.55</v>
@@ -6285,15 +6285,15 @@
         <v>238.333333333333</v>
       </c>
       <c r="I11" s="65" t="s">
-        <v>126</v>
+        <v>93</v>
       </c>
       <c r="J11" s="53" t="n">
         <f aca="false">IF(I11="Win",F11+G11,IF(I11="Push",F11,IF(I11="Loss",0,0)))</f>
-        <v>0</v>
+        <v>238.333333333333</v>
       </c>
       <c r="K11" s="55" t="n">
         <f aca="false">IF(I11="Pending",0,J11-F11)</f>
-        <v>0</v>
+        <v>108.333333333333</v>
       </c>
       <c r="L11" s="66" t="n">
         <v>0.6</v>
@@ -6330,15 +6330,15 @@
         <v>219.173553719008</v>
       </c>
       <c r="I12" s="65" t="s">
-        <v>126</v>
+        <v>93</v>
       </c>
       <c r="J12" s="53" t="n">
         <f aca="false">IF(I12="Win",F12+G12,IF(I12="Push",F12,IF(I12="Loss",0,0)))</f>
-        <v>0</v>
+        <v>219.173553719008</v>
       </c>
       <c r="K12" s="55" t="n">
         <f aca="false">IF(I12="Pending",0,J12-F12)</f>
-        <v>0</v>
+        <v>99.1735537190083</v>
       </c>
       <c r="L12" s="66" t="n">
         <v>0.58</v>
@@ -6415,11 +6415,11 @@
       <c r="I14" s="37"/>
       <c r="J14" s="40" t="n">
         <f aca="false">SUM(J7:J13)</f>
-        <v>533.228511530398</v>
+        <v>701.846509693851</v>
       </c>
       <c r="K14" s="41" t="n">
         <f aca="false">SUM(K7:K13)</f>
-        <v>-216.771488469602</v>
+        <v>-298.153490306149</v>
       </c>
       <c r="L14" s="67" t="n">
         <f aca="false">SUM(L7:L13)</f>
@@ -6438,7 +6438,7 @@
       </c>
       <c r="C17" s="60" t="n">
         <f aca="false">COUNTIF(I7:I13,"Win")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6447,7 +6447,7 @@
       </c>
       <c r="C18" s="60" t="n">
         <f aca="false">COUNTIF(I7:I13,"Loss")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6465,7 +6465,7 @@
       </c>
       <c r="C20" s="60" t="n">
         <f aca="false">COUNTIF(I7:I13,"Pending")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6474,7 +6474,7 @@
       </c>
       <c r="C21" s="61" t="n">
         <f aca="false">IF(COUNTIF(I7:I13,"Win")+COUNTIF(I7:I13,"Loss")=0,"—",COUNTIF(I7:I13,"Win")/(COUNTIF(I7:I13,"Win")+COUNTIF(I7:I13,"Loss")))</f>
-        <v>0.4</v>
+        <v>0.428571428571429</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6492,7 +6492,7 @@
       </c>
       <c r="C23" s="53" t="n">
         <f aca="false">SUM(J7:J13)</f>
-        <v>533.228511530398</v>
+        <v>701.846509693851</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6501,7 +6501,7 @@
       </c>
       <c r="C24" s="55" t="n">
         <f aca="false">SUM(K7:K13)</f>
-        <v>-216.771488469602</v>
+        <v>-298.153490306149</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6510,7 +6510,7 @@
       </c>
       <c r="C25" s="61" t="n">
         <f aca="false">IF(SUM(F7:F13)=0,"—",SUM(K7:K13)/SUM(F7:F13))</f>
-        <v>-0.216771488469602</v>
+        <v>-0.298153490306149</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Settle NASCAR Quaker State 400: 1-6, -$434.51 (Blaney OT win; H2H cashed, basket swept)
- Grade all 7 NASCAR bets in tracker; card SETTLED, tab greyed; balance $4,234.68
- Longshot tracker 0-for-4 (Larson miss); Koepka last live longshot
- Update NASCAR card, account dashboard, index (NASCAR -> Archive); regen PDFs
- Betty settle announcement + manifest; next expected France-Spain Tue

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NqXiXvhRYrGdoae6pGRc4S
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -101,18 +101,21 @@
     <t xml:space="preserve">2026-07-12</t>
   </si>
   <si>
+    <t xml:space="preserve">SETTLED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tab: NASCAR Jul 12 · SETTLED 1-6 (14.3%), -$434.51 · Blaney won in OT after 3h lightning red flag; Wallace P2 stripped (yellow-line)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">World Cup 2026 — Final Four</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jul 14-19</t>
+  </si>
+  <si>
     <t xml:space="preserve">ACTIVE</t>
   </si>
   <si>
-    <t xml:space="preserve">Tab: NASCAR Jul 12 · red-flag lightning delay at lap 109 · finish ~1 AM CT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">World Cup 2026 — Final Four</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jul 14-19</t>
-  </si>
-  <si>
     <t xml:space="preserve">Tab: World Cup 2026 · semis Tue/Wed, final Sun</t>
   </si>
   <si>
@@ -140,9 +143,6 @@
     <t xml:space="preserve">WNBA Sunday Doubleheader</t>
   </si>
   <si>
-    <t xml:space="preserve">SETTLED</t>
-  </si>
-  <si>
     <t xml:space="preserve">Tab: WNBA Jul 12 · SETTLED 3-4 (42.9%), -$298.15 · Fever routed Aces 109-75</t>
   </si>
   <si>
@@ -866,7 +866,7 @@
     <t xml:space="preserve">TEST 4 — NASCAR QUAKER STATE 400 · ECHOPARK SPEEDWAY (ATLANTA) · JULY 12, 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">STATUS: ACTIVE — red-flagged (lightning) at lap 109/260; finish expected ~1 AM CT</t>
+    <t xml:space="preserve">STATUS: SETTLED — Blaney won in OT ~12:55 AM CT Mon after 3h lightning red flag · card 1-6, net -$434.51</t>
   </si>
   <si>
     <t xml:space="preserve">Race ~7:00 PM ET on TNT · Source: nascar-jul12-betting-card.html · Odds: Covers/VSiN/CBS (FanDuel) consensus, Sunday PM</t>
@@ -884,7 +884,7 @@
     <t xml:space="preserve">Matchup</t>
   </si>
   <si>
-    <t xml:space="preserve">7 top-10s in last 8 here; 1 wreck in 16 starts vs Byron's 4 in 14</t>
+    <t xml:space="preserve">7 top-10s in last 8 here; 1 wreck in 16 starts vs Byron's 4 in 14 · WIN — Blaney won the race outright (OT, ~12:55 AM CT Mon); H2H over Byron clinched</t>
   </si>
   <si>
     <t xml:space="preserve">Daniel Suarez Top-5</t>
@@ -893,7 +893,7 @@
     <t xml:space="preserve">Finishing position prop</t>
   </si>
   <si>
-    <t xml:space="preserve">Top-5 in 4 of last 6 Atlanta races; biggest % edge on card</t>
+    <t xml:space="preserve">Top-5 in 4 of last 6 Atlanta races; biggest % edge on card · LOSS — official top 5: Blaney, Bell, Hocevar, Gibbs, E. Jones; Suárez outside top 5</t>
   </si>
   <si>
     <t xml:space="preserve">Chase Elliott to Win</t>
@@ -902,31 +902,31 @@
     <t xml:space="preserve">Outright winner</t>
   </si>
   <si>
-    <t xml:space="preserve">Defending race winner, Georgia native, Chevy won 4 of last 5 here</t>
+    <t xml:space="preserve">Defending race winner, Georgia native, Chevy won 4 of last 5 here · LOSS — Elliott did not win (Blaney P1)</t>
   </si>
   <si>
     <t xml:space="preserve">Carson Hocevar to Win</t>
   </si>
   <si>
-    <t xml:space="preserve">3 straight Atlanta top-10s; elite drafter</t>
+    <t xml:space="preserve">3 straight Atlanta top-10s; elite drafter · LOSS — Hocevar P3; closest of the winner basket</t>
   </si>
   <si>
     <t xml:space="preserve">Brad Keselowski to Win</t>
   </si>
   <si>
-    <t xml:space="preserve">2 Atlanta wins, 6 top-3s; CBS model top pick; RFK form</t>
+    <t xml:space="preserve">2 Atlanta wins, 6 top-3s; CBS model top pick; RFK form · LOSS — Keselowski did not win</t>
   </si>
   <si>
     <t xml:space="preserve">Tyler Reddick to Win</t>
   </si>
   <si>
-    <t xml:space="preserve">Drafting ace; Toyota gambled on race trim over qualifying</t>
+    <t xml:space="preserve">Drafting ace; Toyota gambled on race trim over qualifying · LOSS — Reddick did not win (P8 per post-race reports)</t>
   </si>
   <si>
     <t xml:space="preserve">Kyle Larson to Win (LONGSHOT)</t>
   </si>
   <si>
-    <t xml:space="preserve">Mandatory longshot — best driver at his longest price; P3 start</t>
+    <t xml:space="preserve">Mandatory longshot — best driver at his longest price; P3 start · LOSS — Larson did not win; longshot record now 0-for-4</t>
   </si>
   <si>
     <t xml:space="preserve">Best-Case P/L (basket excl.)</t>
@@ -2253,7 +2253,7 @@
       </c>
       <c r="B6" s="7" t="n">
         <f aca="false">H23</f>
-        <v>-330.81085941033</v>
+        <v>-765.324133746613</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2262,7 +2262,7 @@
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">B5+B6</f>
-        <v>4669.18914058967</v>
+        <v>4234.67586625339</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">F23</f>
-        <v>2600</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2280,7 +2280,7 @@
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">B7-B8</f>
-        <v>2069.18914058967</v>
+        <v>2634.67586625339</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="B10" s="10" t="str">
         <f aca="false">COUNTIF(D16:D22,"ACTIVE")&amp;" of 4 max"</f>
-        <v>3 of 4 max</v>
+        <v>2 of 4 max</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2356,19 +2356,19 @@
       </c>
       <c r="F16" s="16" t="n">
         <f aca="false">SUMIF('NASCAR Jul 12'!I7:I13,"Pending",'NASCAR Jul 12'!F7:F13)</f>
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="G16" s="17" t="n">
         <f aca="false">SUM('NASCAR Jul 12'!J7:J13)</f>
-        <v>0</v>
+        <v>565.486725663717</v>
       </c>
       <c r="H16" s="18" t="n">
         <f aca="false">SUM('NASCAR Jul 12'!K7:K13)</f>
-        <v>0</v>
+        <v>-434.513274336283</v>
       </c>
       <c r="I16" s="19" t="n">
         <f aca="false">B5+H16</f>
-        <v>5000</v>
+        <v>4565.48672566372</v>
       </c>
       <c r="J16" s="20" t="s">
         <v>25</v>
@@ -2385,7 +2385,7 @@
         <v>27</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="E17" s="16" t="n">
         <f aca="false">SUM('World Cup 2026'!F7:F13)</f>
@@ -2405,10 +2405,10 @@
       </c>
       <c r="I17" s="19" t="n">
         <f aca="false">I16+H17</f>
-        <v>5000</v>
+        <v>4565.48672566372</v>
       </c>
       <c r="J17" s="20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2416,13 +2416,13 @@
         <v>6</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="E18" s="16" t="n">
         <f aca="false">SUM('The Open'!F7:F12)</f>
@@ -2442,10 +2442,10 @@
       </c>
       <c r="I18" s="19" t="n">
         <f aca="false">I17+H18</f>
-        <v>5000</v>
+        <v>4565.48672566372</v>
       </c>
       <c r="J18" s="20" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2453,13 +2453,13 @@
         <v>7</v>
       </c>
       <c r="B19" s="22" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C19" s="21" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E19" s="24" t="n">
         <v>0</v>
@@ -2475,10 +2475,10 @@
       </c>
       <c r="I19" s="27" t="n">
         <f aca="false">I18+H19</f>
-        <v>5000</v>
+        <v>4565.48672566372</v>
       </c>
       <c r="J19" s="28" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2486,13 +2486,13 @@
         <v>5</v>
       </c>
       <c r="B20" s="30" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C20" s="29" t="s">
         <v>23</v>
       </c>
       <c r="D20" s="31" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="E20" s="32" t="n">
         <f aca="false">SUM('WNBA Jul 12'!F7:F13)</f>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="I20" s="35" t="n">
         <f aca="false">I19+H20</f>
-        <v>4701.84650969385</v>
+        <v>4267.33323535757</v>
       </c>
       <c r="J20" s="36" t="s">
         <v>38</v>
@@ -2529,7 +2529,7 @@
         <v>23</v>
       </c>
       <c r="D21" s="31" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="E21" s="32" t="n">
         <f aca="false">SUM('MLB Jul 12'!F7:F14)</f>
@@ -2549,7 +2549,7 @@
       </c>
       <c r="I21" s="35" t="n">
         <f aca="false">I20+H21</f>
-        <v>4504.07876775837</v>
+        <v>4069.56549342208</v>
       </c>
       <c r="J21" s="36" t="s">
         <v>40</v>
@@ -2566,7 +2566,7 @@
         <v>42</v>
       </c>
       <c r="D22" s="31" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="E22" s="32" t="n">
         <f aca="false">SUM('UFC 329'!F7:F15)</f>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="I22" s="35" t="n">
         <f aca="false">I21+H22</f>
-        <v>4669.18914058967</v>
+        <v>4234.67586625339</v>
       </c>
       <c r="J22" s="36" t="s">
         <v>43</v>
@@ -2605,15 +2605,15 @@
       </c>
       <c r="F23" s="39" t="n">
         <f aca="false">SUM(F16:F22)</f>
-        <v>2600</v>
+        <v>1600</v>
       </c>
       <c r="G23" s="40" t="n">
         <f aca="false">SUM(G16:G22)</f>
-        <v>2719.18914058967</v>
+        <v>3284.67586625339</v>
       </c>
       <c r="H23" s="41" t="n">
         <f aca="false">SUM(H16:H22)</f>
-        <v>-330.81085941033</v>
+        <v>-765.324133746613</v>
       </c>
       <c r="I23" s="37"/>
       <c r="J23" s="37"/>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="E29" s="10" t="str">
         <f aca="false">IF('NASCAR Jul 12'!I13="Win","HIT",IF('NASCAR Jul 12'!I13="Loss","MISS","Pending"))</f>
-        <v>Pending</v>
+        <v>MISS</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2755,7 +2755,7 @@
       <c r="D33" s="37"/>
       <c r="E33" s="45" t="str">
         <f aca="false">IF(COUNTIF(E27:E32,"HIT")+COUNTIF(E27:E32,"MISS")=0,"—",COUNTIF(E27:E32,"HIT")&amp;"-for-"&amp;(COUNTIF(E27:E32,"HIT")+COUNTIF(E27:E32,"MISS"))&amp;" ("&amp;TEXT(COUNTIF(E27:E32,"HIT")/(COUNTIF(E27:E32,"HIT")+COUNTIF(E27:E32,"MISS")),"0%")&amp;")")</f>
-        <v>0-for-3 (0%)</v>
+        <v>0-for-4 (0%)</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5023,7 +5023,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF1B7A3D"/>
+    <tabColor rgb="FF808080"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M29"/>
@@ -5133,15 +5133,15 @@
         <v>565.486725663717</v>
       </c>
       <c r="I7" s="65" t="s">
-        <v>126</v>
+        <v>93</v>
       </c>
       <c r="J7" s="53" t="n">
         <f aca="false">IF(I7="Win",F7+G7,IF(I7="Push",F7,IF(I7="Loss",0,0)))</f>
-        <v>0</v>
+        <v>565.486725663717</v>
       </c>
       <c r="K7" s="55" t="n">
         <f aca="false">IF(I7="Pending",0,J7-F7)</f>
-        <v>0</v>
+        <v>265.486725663717</v>
       </c>
       <c r="L7" s="66" t="n">
         <v>0.58</v>
@@ -5178,7 +5178,7 @@
         <v>1112</v>
       </c>
       <c r="I8" s="65" t="s">
-        <v>126</v>
+        <v>101</v>
       </c>
       <c r="J8" s="53" t="n">
         <f aca="false">IF(I8="Win",F8+G8,IF(I8="Push",F8,IF(I8="Loss",0,0)))</f>
@@ -5186,7 +5186,7 @@
       </c>
       <c r="K8" s="55" t="n">
         <f aca="false">IF(I8="Pending",0,J8-F8)</f>
-        <v>0</v>
+        <v>-200</v>
       </c>
       <c r="L8" s="66" t="n">
         <v>0.24</v>
@@ -5223,7 +5223,7 @@
         <v>1875</v>
       </c>
       <c r="I9" s="65" t="s">
-        <v>126</v>
+        <v>101</v>
       </c>
       <c r="J9" s="53" t="n">
         <f aca="false">IF(I9="Win",F9+G9,IF(I9="Push",F9,IF(I9="Loss",0,0)))</f>
@@ -5231,7 +5231,7 @@
       </c>
       <c r="K9" s="55" t="n">
         <f aca="false">IF(I9="Pending",0,J9-F9)</f>
-        <v>0</v>
+        <v>-150</v>
       </c>
       <c r="L9" s="66" t="n">
         <v>0.1</v>
@@ -5268,7 +5268,7 @@
         <v>2000.4</v>
       </c>
       <c r="I10" s="65" t="s">
-        <v>126</v>
+        <v>101</v>
       </c>
       <c r="J10" s="53" t="n">
         <f aca="false">IF(I10="Win",F10+G10,IF(I10="Push",F10,IF(I10="Loss",0,0)))</f>
@@ -5276,7 +5276,7 @@
       </c>
       <c r="K10" s="55" t="n">
         <f aca="false">IF(I10="Pending",0,J10-F10)</f>
-        <v>0</v>
+        <v>-120</v>
       </c>
       <c r="L10" s="66" t="n">
         <v>0.08</v>
@@ -5313,7 +5313,7 @@
         <v>1900</v>
       </c>
       <c r="I11" s="65" t="s">
-        <v>126</v>
+        <v>101</v>
       </c>
       <c r="J11" s="53" t="n">
         <f aca="false">IF(I11="Win",F11+G11,IF(I11="Push",F11,IF(I11="Loss",0,0)))</f>
@@ -5321,7 +5321,7 @@
       </c>
       <c r="K11" s="55" t="n">
         <f aca="false">IF(I11="Pending",0,J11-F11)</f>
-        <v>0</v>
+        <v>-100</v>
       </c>
       <c r="L11" s="66" t="n">
         <v>0.07</v>
@@ -5358,7 +5358,7 @@
         <v>1125</v>
       </c>
       <c r="I12" s="65" t="s">
-        <v>126</v>
+        <v>101</v>
       </c>
       <c r="J12" s="53" t="n">
         <f aca="false">IF(I12="Win",F12+G12,IF(I12="Push",F12,IF(I12="Loss",0,0)))</f>
@@ -5366,7 +5366,7 @@
       </c>
       <c r="K12" s="55" t="n">
         <f aca="false">IF(I12="Pending",0,J12-F12)</f>
-        <v>0</v>
+        <v>-90</v>
       </c>
       <c r="L12" s="66" t="n">
         <v>0.08</v>
@@ -5403,7 +5403,7 @@
         <v>800</v>
       </c>
       <c r="I13" s="65" t="s">
-        <v>126</v>
+        <v>101</v>
       </c>
       <c r="J13" s="53" t="n">
         <f aca="false">IF(I13="Win",F13+G13,IF(I13="Push",F13,IF(I13="Loss",0,0)))</f>
@@ -5411,7 +5411,7 @@
       </c>
       <c r="K13" s="55" t="n">
         <f aca="false">IF(I13="Pending",0,J13-F13)</f>
-        <v>0</v>
+        <v>-40</v>
       </c>
       <c r="L13" s="66" t="n">
         <v>0.05</v>
@@ -5443,11 +5443,11 @@
       <c r="I14" s="37"/>
       <c r="J14" s="40" t="n">
         <f aca="false">SUM(J7:J13)</f>
-        <v>0</v>
+        <v>565.486725663717</v>
       </c>
       <c r="K14" s="41" t="n">
         <f aca="false">SUM(K7:K13)</f>
-        <v>0</v>
+        <v>-434.513274336283</v>
       </c>
       <c r="L14" s="67" t="n">
         <f aca="false">SUM(L7:L13)</f>
@@ -5466,7 +5466,7 @@
       </c>
       <c r="C17" s="60" t="n">
         <f aca="false">COUNTIF(I7:I13,"Win")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5475,7 +5475,7 @@
       </c>
       <c r="C18" s="60" t="n">
         <f aca="false">COUNTIF(I7:I13,"Loss")</f>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5493,16 +5493,16 @@
       </c>
       <c r="C20" s="60" t="n">
         <f aca="false">COUNTIF(I7:I13,"Pending")</f>
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="C21" s="61" t="str">
+      <c r="C21" s="61" t="n">
         <f aca="false">IF(COUNTIF(I7:I13,"Win")+COUNTIF(I7:I13,"Loss")=0,"—",COUNTIF(I7:I13,"Win")/(COUNTIF(I7:I13,"Win")+COUNTIF(I7:I13,"Loss")))</f>
-        <v>—</v>
+        <v>0.142857142857143</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5520,7 +5520,7 @@
       </c>
       <c r="C23" s="53" t="n">
         <f aca="false">SUM(J7:J13)</f>
-        <v>0</v>
+        <v>565.486725663717</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5529,7 +5529,7 @@
       </c>
       <c r="C24" s="55" t="n">
         <f aca="false">SUM(K7:K13)</f>
-        <v>0</v>
+        <v>-434.513274336283</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5538,7 +5538,7 @@
       </c>
       <c r="C25" s="61" t="n">
         <f aca="false">IF(SUM(F7:F13)=0,"—",SUM(K7:K13)/SUM(F7:F13))</f>
-        <v>0</v>
+        <v>-0.434513274336283</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Derby semis: Rice under 9.5 graded Loss (7 HRs); 1-1 -$6.36; Contreras top seed, 3 horses in final four; Betty u2
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -1281,7 +1281,7 @@
     <t xml:space="preserve">TEST 8 — MLB HOME RUN DERBY · CITIZENS BANK PARK, PHILADELPHIA · JULY 13, 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">STATUS: ACTIVE — LIVE, R1 in progress; longest-HR prop cashed</t>
+    <t xml:space="preserve">STATUS: ACTIVE — 1-1 (−$6.36) · semis: Contreras(1) v Schwarber(4), Walker(2) v Caminero(3)</t>
   </si>
   <si>
     <t xml:space="preserve">8 PM ET / 7 CT on Netflix · Source: cards/hrderby-jul13-betting-card.html · Outrights: DraftKings ~9 AM CT Jul 13 · Props: Action Network / VSiN lines, -110 std price</t>
@@ -1323,7 +1323,7 @@
     <t xml:space="preserve">Ben Rice R1 Over 9.5 HRs</t>
   </si>
   <si>
-    <t xml:space="preserve">Lefty pull power, 330-ft RF corner — VSiN lean</t>
+    <t xml:space="preserve">Lefty pull power, 330-ft RF corner — VSiN lean · RESULT: Rice 7 in R1 — under 9.5 (2 sources)</t>
   </si>
   <si>
     <t xml:space="preserve">Longest HR Over 484.5 ft</t>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="B6" s="7" t="n">
         <f aca="false">H24</f>
-        <v>-651.687770110249</v>
+        <v>-771.687770110249</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">B5+B6</f>
-        <v>4348.31222988975</v>
+        <v>4228.31222988975</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2300,7 +2300,7 @@
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">F24</f>
-        <v>2475</v>
+        <v>2355</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="F16" s="17" t="n">
         <f aca="false">SUMIF('HR Derby'!I7:I13,"Pending",'HR Derby'!F7:F13)</f>
-        <v>875</v>
+        <v>755</v>
       </c>
       <c r="G16" s="17" t="n">
         <f aca="false">SUM('HR Derby'!J7:J13)</f>
@@ -2395,7 +2395,7 @@
       </c>
       <c r="H16" s="17" t="n">
         <f aca="false">SUM('HR Derby'!K7:K13)</f>
-        <v>113.636363636364</v>
+        <v>-6.36363636363637</v>
       </c>
       <c r="I16" s="18"/>
       <c r="J16" s="19"/>
@@ -2654,7 +2654,7 @@
       </c>
       <c r="F24" s="8" t="n">
         <f aca="false">SUM(F16:F23)</f>
-        <v>2475</v>
+        <v>2355</v>
       </c>
       <c r="G24" s="8" t="n">
         <f aca="false">SUM(G16:G23)</f>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="H24" s="8" t="n">
         <f aca="false">SUM(H16:H23)</f>
-        <v>-651.687770110249</v>
+        <v>-771.687770110249</v>
       </c>
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
@@ -7529,7 +7529,7 @@
         <v>229.090909090909</v>
       </c>
       <c r="I11" s="56" t="s">
-        <v>119</v>
+        <v>94</v>
       </c>
       <c r="J11" s="41" t="n">
         <f aca="false">IF(I11="Win",F11+G11,IF(I11="Push",F11,IF(I11="Loss",0,0)))</f>
@@ -7537,7 +7537,7 @@
       </c>
       <c r="K11" s="43" t="n">
         <f aca="false">IF(I11="Pending",0,J11-F11)</f>
-        <v>0</v>
+        <v>-120</v>
       </c>
       <c r="L11" s="72" t="n">
         <v>0.57</v>
@@ -7658,7 +7658,7 @@
       </c>
       <c r="K14" s="8" t="n">
         <f aca="false">SUM(K7:K13)</f>
-        <v>113.636363636364</v>
+        <v>-6.36363636363637</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
The Open Phase 2: deploy reserved $400 as 5 top-10 props (Scheffler/Fleetwood/Rahm/Fitzpatrick/Morikawa); Open now $1,000 at risk
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="785" uniqueCount="465">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="803" uniqueCount="473">
   <si>
     <t xml:space="preserve">BETTING TEST ACCOUNT — ROLL-UP DASHBOARD</t>
   </si>
@@ -1231,13 +1231,13 @@
     <t xml:space="preserve">TEST 6 — THE 154th OPEN CHAMPIONSHIP · ROYAL BIRKDALE · JULY 16-19, 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">STATUS: ACTIVE — first tee Thu Jul 16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source: open2026-betting-card.html · Odds: DraftKings/consensus + Golf Digest, locked Sun Jul 12 · Phase 2 props ($400) added Wed Jul 15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Outright basket is mutually exclusive — max one cashes. Basket coverage ≈ 44%. $600 deployed now; $400 reserved (not yet at risk).</t>
+    <t xml:space="preserve">STATUS: ACTIVE — first tee Thu Jul 16 · $1,000 fully deployed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source: open2026-betting-card.html · Outrights locked Sun Jul 12 · Phase 2 top-10 props deployed Wed Jul 15 (reserved $400 now at risk)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outright basket (rows 7-12) mutually exclusive — max one cashes. Phase 2 = 5 top-10 props (rows 13-17). Full $1,000 now deployed.</t>
   </si>
   <si>
     <t xml:space="preserve">Scottie Scheffler</t>
@@ -1276,13 +1276,37 @@
     <t xml:space="preserve">5 majors, career-long price · counts in longshot record</t>
   </si>
   <si>
-    <t xml:space="preserve">RESERVED — Phase 2 props (Wed)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Top-10s / H2H matchups / make-cut — lines post midweek</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$400 reserved, not yet at risk; converts Wed Jul 15</t>
+    <t xml:space="preserve">Scottie Scheffler Top-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Top-10 finish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">World #1 / +620 favorite; safest of the basket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tommy Fleetwood Top-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Southport native, home links; strong value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jon Rahm Top-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elite wind player; value vs field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matt Fitzpatrick Top-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">English; 6 straight Open cuts made</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collin Morikawa Top-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2021 Open champ, elite ballstriker</t>
   </si>
   <si>
     <t xml:space="preserve">TOTALS (deployed)</t>
@@ -1430,7 +1454,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="11">
+  <numFmts count="13">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
@@ -1441,7 +1465,9 @@
     <numFmt numFmtId="171" formatCode="0%"/>
     <numFmt numFmtId="172" formatCode="0.0&quot; exp. wins&quot;"/>
     <numFmt numFmtId="173" formatCode="0.0"/>
-    <numFmt numFmtId="174" formatCode="0.00&quot; exp. wins&quot;"/>
+    <numFmt numFmtId="174" formatCode="\$#,##0"/>
+    <numFmt numFmtId="175" formatCode="\$#,##0.00"/>
+    <numFmt numFmtId="176" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -1743,7 +1769,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="90">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2040,11 +2066,59 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="176" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="176" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2065,7 +2139,35 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <name val="Arial"/>
@@ -2399,7 +2501,7 @@
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">F25</f>
-        <v>2600</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2408,7 +2510,7 @@
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">B7-B8</f>
-        <v>1159.67586625339</v>
+        <v>759.675866253387</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2551,19 +2653,19 @@
         <v>22</v>
       </c>
       <c r="E18" s="17" t="n">
-        <f aca="false">SUM('The Open'!F7:F12)</f>
-        <v>600</v>
+        <f aca="false">SUM('The Open'!F7:F17)</f>
+        <v>1000</v>
       </c>
       <c r="F18" s="17" t="n">
-        <f aca="false">SUMIF('The Open'!I7:I12,"Pending",'The Open'!F7:F12)</f>
-        <v>600</v>
+        <f aca="false">SUMIF('The Open'!I7:I17,"Pending",'The Open'!F7:F17)</f>
+        <v>1000</v>
       </c>
       <c r="G18" s="17" t="n">
-        <f aca="false">SUM('The Open'!J7:J12)</f>
+        <f aca="false">SUM('The Open'!J7:J17)</f>
         <v>0</v>
       </c>
       <c r="H18" s="17" t="n">
-        <f aca="false">SUM('The Open'!K7:K12)</f>
+        <f aca="false">SUM('The Open'!K7:K17)</f>
         <v>0</v>
       </c>
       <c r="I18" s="18"/>
@@ -2783,11 +2885,11 @@
       </c>
       <c r="E25" s="8" t="n">
         <f aca="false">SUM(E16:E24)</f>
-        <v>7650</v>
+        <v>8050</v>
       </c>
       <c r="F25" s="8" t="n">
         <f aca="false">SUM(F16:F24)</f>
-        <v>2600</v>
+        <v>3000</v>
       </c>
       <c r="G25" s="8" t="n">
         <f aca="false">SUM(G16:G24)</f>
@@ -3128,20 +3230,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="35" t="s">
-        <v>442</v>
-      </c>
-      <c r="H1" s="77" t="s">
-        <v>443</v>
+        <v>450</v>
+      </c>
+      <c r="H1" s="89" t="s">
+        <v>451</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>444</v>
+        <v>452</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>445</v>
+        <v>453</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3195,10 +3297,10 @@
         <v>1</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
       <c r="C7" s="32" t="s">
-        <v>447</v>
+        <v>455</v>
       </c>
       <c r="D7" s="33" t="s">
         <v>378</v>
@@ -3232,7 +3334,7 @@
         <v>0.57</v>
       </c>
       <c r="M7" s="62" t="s">
-        <v>448</v>
+        <v>456</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3240,10 +3342,10 @@
         <v>2</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>449</v>
+        <v>457</v>
       </c>
       <c r="C8" s="32" t="s">
-        <v>450</v>
+        <v>458</v>
       </c>
       <c r="D8" s="33" t="s">
         <v>179</v>
@@ -3277,7 +3379,7 @@
         <v>0.54</v>
       </c>
       <c r="M8" s="62" t="s">
-        <v>451</v>
+        <v>459</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3285,10 +3387,10 @@
         <v>3</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>452</v>
+        <v>460</v>
       </c>
       <c r="C9" s="32" t="s">
-        <v>453</v>
+        <v>461</v>
       </c>
       <c r="D9" s="33" t="s">
         <v>179</v>
@@ -3322,7 +3424,7 @@
         <v>0.55</v>
       </c>
       <c r="M9" s="62" t="s">
-        <v>454</v>
+        <v>462</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3330,7 +3432,7 @@
         <v>4</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>455</v>
+        <v>463</v>
       </c>
       <c r="C10" s="32" t="s">
         <v>393</v>
@@ -3367,7 +3469,7 @@
         <v>0.54</v>
       </c>
       <c r="M10" s="62" t="s">
-        <v>456</v>
+        <v>464</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3375,10 +3477,10 @@
         <v>5</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>457</v>
+        <v>465</v>
       </c>
       <c r="C11" s="32" t="s">
-        <v>458</v>
+        <v>466</v>
       </c>
       <c r="D11" s="33" t="s">
         <v>89</v>
@@ -3412,7 +3514,7 @@
         <v>0.58</v>
       </c>
       <c r="M11" s="62" t="s">
-        <v>459</v>
+        <v>467</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3420,10 +3522,10 @@
         <v>6</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>460</v>
+        <v>468</v>
       </c>
       <c r="C12" s="32" t="s">
-        <v>461</v>
+        <v>469</v>
       </c>
       <c r="D12" s="33" t="s">
         <v>378</v>
@@ -3457,7 +3559,7 @@
         <v>0.52</v>
       </c>
       <c r="M12" s="62" t="s">
-        <v>462</v>
+        <v>470</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3468,7 +3570,7 @@
         <v>395</v>
       </c>
       <c r="C13" s="32" t="s">
-        <v>463</v>
+        <v>471</v>
       </c>
       <c r="D13" s="33" t="s">
         <v>117</v>
@@ -3502,7 +3604,7 @@
         <v>0.1</v>
       </c>
       <c r="M13" s="62" t="s">
-        <v>464</v>
+        <v>472</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7684,7 +7786,7 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="74" t="n">
+      <c r="A13" s="20" t="n">
         <v>7</v>
       </c>
       <c r="B13" s="21" t="s">
@@ -7693,77 +7795,252 @@
       <c r="C13" s="74" t="s">
         <v>416</v>
       </c>
-      <c r="D13" s="74" t="s">
-        <v>63</v>
-      </c>
-      <c r="E13" s="74"/>
-      <c r="F13" s="74"/>
-      <c r="G13" s="74"/>
-      <c r="H13" s="74"/>
-      <c r="I13" s="74"/>
-      <c r="J13" s="74"/>
-      <c r="K13" s="74"/>
-      <c r="L13" s="74"/>
-      <c r="M13" s="74" t="s">
+      <c r="D13" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="E13" s="75" t="n">
+        <v>-146</v>
+      </c>
+      <c r="F13" s="76" t="n">
+        <v>120</v>
+      </c>
+      <c r="G13" s="77" t="n">
+        <f aca="false">IF(E13&gt;0,F13*E13/100,F13*100/ABS(E13))</f>
+        <v>82.1917808219178</v>
+      </c>
+      <c r="H13" s="77" t="n">
+        <f aca="false">F13+G13</f>
+        <v>202.191780821918</v>
+      </c>
+      <c r="I13" s="57" t="s">
+        <v>123</v>
+      </c>
+      <c r="J13" s="77" t="n">
+        <f aca="false">IF(I13="Win",F13+G13,IF(I13="Push",F13,IF(I13="Loss",0,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="K13" s="78" t="n">
+        <f aca="false">IF(I13="Pending",0,J13-F13)</f>
+        <v>0</v>
+      </c>
+      <c r="L13" s="79" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="M13" s="80" t="s">
         <v>417</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="63"/>
-      <c r="B14" s="64" t="s">
+      <c r="A14" s="33" t="n">
+        <v>8</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>418</v>
       </c>
-      <c r="C14" s="63"/>
-      <c r="D14" s="63"/>
-      <c r="E14" s="63"/>
-      <c r="F14" s="48" t="n">
-        <f aca="false">SUM(F7:F13)</f>
-        <v>600</v>
-      </c>
-      <c r="G14" s="49" t="n">
-        <f aca="false">SUM(G7:G12)</f>
-        <v>10160</v>
-      </c>
-      <c r="H14" s="49" t="n">
-        <f aca="false">SUM(H7:H12)</f>
-        <v>10760</v>
-      </c>
-      <c r="I14" s="63"/>
-      <c r="J14" s="49" t="n">
-        <f aca="false">SUM(J7:J12)</f>
-        <v>0</v>
-      </c>
-      <c r="K14" s="50" t="n">
-        <f aca="false">SUM(K7:K12)</f>
-        <v>0</v>
-      </c>
-      <c r="L14" s="75" t="n">
-        <f aca="false">SUM(L7:L12)</f>
-        <v>0.445</v>
-      </c>
-      <c r="M14" s="63"/>
+      <c r="C14" s="32" t="s">
+        <v>416</v>
+      </c>
+      <c r="D14" s="33" t="s">
+        <v>94</v>
+      </c>
+      <c r="E14" s="39" t="n">
+        <v>158</v>
+      </c>
+      <c r="F14" s="81" t="n">
+        <v>90</v>
+      </c>
+      <c r="G14" s="82" t="n">
+        <f aca="false">IF(E14&gt;0,F14*E14/100,F14*100/ABS(E14))</f>
+        <v>142.2</v>
+      </c>
+      <c r="H14" s="82" t="n">
+        <f aca="false">F14+G14</f>
+        <v>232.2</v>
+      </c>
+      <c r="I14" s="57" t="s">
+        <v>123</v>
+      </c>
+      <c r="J14" s="82" t="n">
+        <f aca="false">IF(I14="Win",F14+G14,IF(I14="Push",F14,IF(I14="Loss",0,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="K14" s="83" t="n">
+        <f aca="false">IF(I14="Pending",0,J14-F14)</f>
+        <v>0</v>
+      </c>
+      <c r="L14" s="73" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="M14" s="62" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="33" t="n">
+        <v>9</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>420</v>
+      </c>
+      <c r="C15" s="32" t="s">
+        <v>416</v>
+      </c>
+      <c r="D15" s="33" t="s">
+        <v>94</v>
+      </c>
+      <c r="E15" s="39" t="n">
+        <v>172</v>
+      </c>
+      <c r="F15" s="81" t="n">
+        <v>80</v>
+      </c>
+      <c r="G15" s="82" t="n">
+        <f aca="false">IF(E15&gt;0,F15*E15/100,F15*100/ABS(E15))</f>
+        <v>137.6</v>
+      </c>
+      <c r="H15" s="82" t="n">
+        <f aca="false">F15+G15</f>
+        <v>217.6</v>
+      </c>
+      <c r="I15" s="57" t="s">
+        <v>123</v>
+      </c>
+      <c r="J15" s="82" t="n">
+        <f aca="false">IF(I15="Win",F15+G15,IF(I15="Push",F15,IF(I15="Loss",0,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="K15" s="83" t="n">
+        <f aca="false">IF(I15="Pending",0,J15-F15)</f>
+        <v>0</v>
+      </c>
+      <c r="L15" s="73" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="M15" s="62" t="s">
+        <v>421</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="4" t="s">
-        <v>119</v>
+      <c r="A16" s="33" t="n">
+        <v>10</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="C16" s="32" t="s">
+        <v>416</v>
+      </c>
+      <c r="D16" s="33" t="s">
+        <v>94</v>
+      </c>
+      <c r="E16" s="39" t="n">
+        <v>164</v>
+      </c>
+      <c r="F16" s="81" t="n">
+        <v>70</v>
+      </c>
+      <c r="G16" s="82" t="n">
+        <f aca="false">IF(E16&gt;0,F16*E16/100,F16*100/ABS(E16))</f>
+        <v>114.8</v>
+      </c>
+      <c r="H16" s="82" t="n">
+        <f aca="false">F16+G16</f>
+        <v>184.8</v>
+      </c>
+      <c r="I16" s="57" t="s">
+        <v>123</v>
+      </c>
+      <c r="J16" s="82" t="n">
+        <f aca="false">IF(I16="Win",F16+G16,IF(I16="Push",F16,IF(I16="Loss",0,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="K16" s="83" t="n">
+        <f aca="false">IF(I16="Pending",0,J16-F16)</f>
+        <v>0</v>
+      </c>
+      <c r="L16" s="73" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="M16" s="62" t="s">
+        <v>423</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="33" t="n">
+        <v>11</v>
+      </c>
       <c r="B17" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="C17" s="51" t="n">
-        <f aca="false">COUNTIF(I7:I12,"Win")</f>
-        <v>0</v>
+        <v>424</v>
+      </c>
+      <c r="C17" s="84" t="s">
+        <v>416</v>
+      </c>
+      <c r="D17" s="33" t="s">
+        <v>94</v>
+      </c>
+      <c r="E17" s="39" t="n">
+        <v>280</v>
+      </c>
+      <c r="F17" s="81" t="n">
+        <v>40</v>
+      </c>
+      <c r="G17" s="82" t="n">
+        <f aca="false">IF(E17&gt;0,F17*E17/100,F17*100/ABS(E17))</f>
+        <v>112</v>
+      </c>
+      <c r="H17" s="82" t="n">
+        <f aca="false">F17+G17</f>
+        <v>152</v>
+      </c>
+      <c r="I17" s="57" t="s">
+        <v>123</v>
+      </c>
+      <c r="J17" s="82" t="n">
+        <f aca="false">IF(I17="Win",F17+G17,IF(I17="Push",F17,IF(I17="Loss",0,0)))</f>
+        <v>0</v>
+      </c>
+      <c r="K17" s="83" t="n">
+        <f aca="false">IF(I17="Pending",0,J17-F17)</f>
+        <v>0</v>
+      </c>
+      <c r="L17" s="73" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M17" s="62" t="s">
+        <v>425</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="5" t="s">
-        <v>121</v>
+      <c r="B18" s="85" t="s">
+        <v>426</v>
       </c>
       <c r="C18" s="51" t="n">
         <f aca="false">COUNTIF(I7:I12,"Loss")</f>
         <v>0</v>
+      </c>
+      <c r="F18" s="86" t="n">
+        <f aca="false">SUM(F7:F17)</f>
+        <v>1000</v>
+      </c>
+      <c r="G18" s="86" t="n">
+        <f aca="false">SUM(G7:G17)</f>
+        <v>10748.7917808219</v>
+      </c>
+      <c r="H18" s="86" t="n">
+        <f aca="false">SUM(H7:H17)</f>
+        <v>11748.7917808219</v>
+      </c>
+      <c r="J18" s="86" t="n">
+        <f aca="false">SUM(J7:J17)</f>
+        <v>0</v>
+      </c>
+      <c r="K18" s="86" t="n">
+        <f aca="false">SUM(K7:K17)</f>
+        <v>0</v>
+      </c>
+      <c r="L18" s="87" t="n">
+        <f aca="false">SUM(L7:L17)</f>
+        <v>2.645</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7786,7 +8063,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="5" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="C21" s="34" t="n">
         <f aca="false">SUM(F7:F12)</f>
@@ -7813,7 +8090,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="5" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
       <c r="C24" s="52" t="n">
         <f aca="false">SUM(L7:L12)</f>
@@ -7837,8 +8114,20 @@
       <formula>AND(ISNUMBER(C23),C23&lt;0)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <conditionalFormatting sqref="K7:K18">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>AND(ISNUMBER(K7),K7&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+      <formula>AND(ISNUMBER(K7),K7&lt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I7:I12" type="list">
+      <formula1>"Pending,Win,Loss,Push"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I13:I17" type="list">
       <formula1>"Pending,Win,Loss,Push"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -7878,20 +8167,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="35" t="s">
-        <v>421</v>
-      </c>
-      <c r="H1" s="76" t="s">
-        <v>422</v>
+        <v>429</v>
+      </c>
+      <c r="H1" s="88" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>423</v>
+        <v>431</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>424</v>
+        <v>432</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7945,7 +8234,7 @@
         <v>1</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>425</v>
+        <v>433</v>
       </c>
       <c r="C7" s="32" t="s">
         <v>287</v>
@@ -7982,7 +8271,7 @@
         <v>0.27</v>
       </c>
       <c r="M7" s="62" t="s">
-        <v>426</v>
+        <v>434</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7990,7 +8279,7 @@
         <v>2</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>427</v>
+        <v>435</v>
       </c>
       <c r="C8" s="32" t="s">
         <v>287</v>
@@ -8027,7 +8316,7 @@
         <v>0.18</v>
       </c>
       <c r="M8" s="62" t="s">
-        <v>428</v>
+        <v>436</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8035,10 +8324,10 @@
         <v>3</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>429</v>
+        <v>437</v>
       </c>
       <c r="C9" s="32" t="s">
-        <v>430</v>
+        <v>438</v>
       </c>
       <c r="D9" s="33" t="s">
         <v>94</v>
@@ -8072,7 +8361,7 @@
         <v>0.6</v>
       </c>
       <c r="M9" s="62" t="s">
-        <v>431</v>
+        <v>439</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8080,10 +8369,10 @@
         <v>4</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>432</v>
+        <v>440</v>
       </c>
       <c r="C10" s="32" t="s">
-        <v>433</v>
+        <v>441</v>
       </c>
       <c r="D10" s="33" t="s">
         <v>94</v>
@@ -8117,7 +8406,7 @@
         <v>0.58</v>
       </c>
       <c r="M10" s="62" t="s">
-        <v>434</v>
+        <v>442</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8125,10 +8414,10 @@
         <v>5</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>435</v>
+        <v>443</v>
       </c>
       <c r="C11" s="32" t="s">
-        <v>430</v>
+        <v>438</v>
       </c>
       <c r="D11" s="33" t="s">
         <v>94</v>
@@ -8162,7 +8451,7 @@
         <v>0.57</v>
       </c>
       <c r="M11" s="62" t="s">
-        <v>436</v>
+        <v>444</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8170,10 +8459,10 @@
         <v>6</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>437</v>
+        <v>445</v>
       </c>
       <c r="C12" s="32" t="s">
-        <v>438</v>
+        <v>446</v>
       </c>
       <c r="D12" s="33" t="s">
         <v>94</v>
@@ -8207,7 +8496,7 @@
         <v>0.56</v>
       </c>
       <c r="M12" s="62" t="s">
-        <v>439</v>
+        <v>447</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8215,7 +8504,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>440</v>
+        <v>448</v>
       </c>
       <c r="C13" s="32" t="s">
         <v>287</v>
@@ -8252,7 +8541,7 @@
         <v>0.07</v>
       </c>
       <c r="M13" s="62" t="s">
-        <v>441</v>
+        <v>449</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Open R2 live update 4:10 PM UK Fri: both 62 totals verified — TSN confirms Herbert finished -8 (62), leads after missed par putt on the last (9-under thru 16); Burns total -5 (62, holed greenside bunker shot at 18, first birdie there all day). Suber clubhouse -6, Cam Young 67-67 -6, McIlroy 67 safe at -3. CUT ALARM: Golf Monthly reports Fitzpatrick +4 with 3 to play, in danger of missing cut (~+1) — $150 of card exposure, one-source pending confirmation next check. Morikawa no fresher than -5 thru 9; Koepka no in-play number (E). Scheffler/Rahm/Fleetwood on course ~1 hr, no syndicated numbers yet. Banner, dashboard tile, tracker status + PDFs refreshed; rebased onto Rugby-finalize commit (at-risk now $1,550). No grading — settles Sunday.
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KN6cZWxSbBCs8xL5WQXgx6
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -1229,7 +1229,7 @@
     <t xml:space="preserve">TEST 6 — THE 154th OPEN CHAMPIONSHIP · ROYAL BIRKDALE · JULY 16-19, 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">STATUS: ACTIVE — R2 IN PROGRESS Fri Jul 17 (3:10 PM UK): TWO record 62s — Herbert leads -8; The Open official feed: "Sam Burns also cards an impressive 62 at Royal Birkdale" (Yahoo headline: both tie record for lowest major score ever; Burns total pending). Suber clubhouse -6. Morikawa no fresher number (last -5 thru 9, best on card). Koepka/Fitzpatrick no in-play numbers (E / +2 overnight, cut watch). Cut ~+1 (Yahoo 53%, Data Golf 50.9%). Scheffler off 3:04, Rahm/Fleetwood off 3:15 PM UK — $760 of card on course. Grade Sunday night only.</t>
+    <t xml:space="preserve">STATUS: ACTIVE — R2 IN PROGRESS Fri Jul 17 (4:10 PM UK): Both 62 totals now verified — TSN: Herbert finished -8 (62) and leads (9-under thru 16, missed par putt on 18); Burns total -5 (62, holed greenside bunker shot at 18). Suber clubhouse -6; Cam Young 67-67 -6. CUT ALARM: Golf Monthly reports Fitzpatrick +4 with 3 to play, in danger of missing cut (~+1) — one-source, confirm next check. Morikawa no fresher than -5 thru 9. Koepka no in-play number (E overnight). Scheffler (-2), Rahm/Fleetwood (-1) on course since 3:04/3:15 PM UK, no syndicated numbers yet. Grade Sunday night only.</t>
   </si>
   <si>
     <t xml:space="preserve">Source: open2026-betting-card.html · Outrights locked Sun Jul 12 · Phase 2 top-10 props deployed Wed Jul 15 (reserved $400 now at risk)</t>
@@ -1494,7 +1494,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="13">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
@@ -1505,9 +1505,6 @@
     <numFmt numFmtId="171" formatCode="0%"/>
     <numFmt numFmtId="172" formatCode="0.0&quot; exp. wins&quot;"/>
     <numFmt numFmtId="173" formatCode="0.0"/>
-    <numFmt numFmtId="174" formatCode="\$#,##0"/>
-    <numFmt numFmtId="175" formatCode="\$#,##0.00"/>
-    <numFmt numFmtId="176" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -1815,7 +1812,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="85">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2092,10 +2089,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="170" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2156,36 +2149,8 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="14" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="14" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="174" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="175" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="176" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="175" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2197,35 +2162,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <charset val="1"/>
-        <family val="0"/>
-        <b val="1"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <charset val="1"/>
-        <family val="0"/>
-        <b val="1"/>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <name val="Arial"/>
@@ -3295,7 +3232,7 @@
       <c r="A1" s="31" t="s">
         <v>449</v>
       </c>
-      <c r="H1" s="84" t="s">
+      <c r="H1" s="83" t="s">
         <v>450</v>
       </c>
     </row>
@@ -3393,7 +3330,7 @@
         <f aca="false">IF(I7="Pending",0,J7-F7)</f>
         <v>-185</v>
       </c>
-      <c r="L7" s="70" t="n">
+      <c r="L7" s="69" t="n">
         <v>0.57</v>
       </c>
       <c r="M7" s="58" t="s">
@@ -3438,7 +3375,7 @@
         <f aca="false">IF(I8="Pending",0,J8-F8)</f>
         <v>-175</v>
       </c>
-      <c r="L8" s="70" t="n">
+      <c r="L8" s="69" t="n">
         <v>0.54</v>
       </c>
       <c r="M8" s="58" t="s">
@@ -3483,7 +3420,7 @@
         <f aca="false">IF(I9="Pending",0,J9-F9)</f>
         <v>145.454545454546</v>
       </c>
-      <c r="L9" s="70" t="n">
+      <c r="L9" s="69" t="n">
         <v>0.55</v>
       </c>
       <c r="M9" s="58" t="s">
@@ -3528,7 +3465,7 @@
         <f aca="false">IF(I10="Pending",0,J10-F10)</f>
         <v>-150</v>
       </c>
-      <c r="L10" s="70" t="n">
+      <c r="L10" s="69" t="n">
         <v>0.54</v>
       </c>
       <c r="M10" s="58" t="s">
@@ -3573,7 +3510,7 @@
         <f aca="false">IF(I11="Pending",0,J11-F11)</f>
         <v>107.692307692308</v>
       </c>
-      <c r="L11" s="70" t="n">
+      <c r="L11" s="69" t="n">
         <v>0.58</v>
       </c>
       <c r="M11" s="58" t="s">
@@ -3618,7 +3555,7 @@
         <f aca="false">IF(I12="Pending",0,J12-F12)</f>
         <v>-115</v>
       </c>
-      <c r="L12" s="70" t="n">
+      <c r="L12" s="69" t="n">
         <v>0.52</v>
       </c>
       <c r="M12" s="58" t="s">
@@ -3663,7 +3600,7 @@
         <f aca="false">IF(I13="Pending",0,J13-F13)</f>
         <v>-75</v>
       </c>
-      <c r="L13" s="70" t="n">
+      <c r="L13" s="69" t="n">
         <v>0.1</v>
       </c>
       <c r="M13" s="58" t="s">
@@ -3729,44 +3666,44 @@
   <dimension ref="A1:M10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="50"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="85" t="s">
+    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="31" t="s">
         <v>472</v>
       </c>
-      <c r="H1" s="86" t="s">
+      <c r="H1" s="84" t="s">
         <v>473</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="87" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>474</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="87" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>475</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="88" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
         <v>12</v>
       </c>
@@ -3807,7 +3744,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="29" t="n">
         <v>1</v>
       </c>
@@ -3823,36 +3760,36 @@
       <c r="E7" s="35" t="n">
         <v>-111</v>
       </c>
-      <c r="F7" s="89" t="n">
+      <c r="F7" s="36" t="n">
         <v>340</v>
       </c>
-      <c r="G7" s="90" t="n">
+      <c r="G7" s="37" t="n">
         <f aca="false">IF(E7&gt;0,F7*E7/100,F7*100/ABS(E7))</f>
         <v>306.306306306306</v>
       </c>
-      <c r="H7" s="90" t="n">
+      <c r="H7" s="37" t="n">
         <f aca="false">F7+G7</f>
         <v>646.306306306306</v>
       </c>
       <c r="I7" s="53" t="s">
         <v>121</v>
       </c>
-      <c r="J7" s="90" t="n">
+      <c r="J7" s="37" t="n">
         <f aca="false">IF(I7="Win",F7+G7,IF(I7="Push",F7,IF(I7="Loss",0,0)))</f>
         <v>0</v>
       </c>
-      <c r="K7" s="91" t="n">
+      <c r="K7" s="39" t="n">
         <f aca="false">IF(I7="Pending",0,J7-F7)</f>
         <v>0</v>
       </c>
-      <c r="L7" s="70" t="n">
+      <c r="L7" s="69" t="n">
         <v>0.6</v>
       </c>
       <c r="M7" s="58" t="s">
         <v>479</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="29" t="n">
         <v>2</v>
       </c>
@@ -3868,36 +3805,36 @@
       <c r="E8" s="35" t="n">
         <v>-110</v>
       </c>
-      <c r="F8" s="89" t="n">
+      <c r="F8" s="36" t="n">
         <v>150</v>
       </c>
-      <c r="G8" s="90" t="n">
+      <c r="G8" s="37" t="n">
         <f aca="false">IF(E8&gt;0,F8*E8/100,F8*100/ABS(E8))</f>
         <v>136.363636363636</v>
       </c>
-      <c r="H8" s="90" t="n">
+      <c r="H8" s="37" t="n">
         <f aca="false">F8+G8</f>
         <v>286.363636363636</v>
       </c>
       <c r="I8" s="53" t="s">
         <v>121</v>
       </c>
-      <c r="J8" s="90" t="n">
+      <c r="J8" s="37" t="n">
         <f aca="false">IF(I8="Win",F8+G8,IF(I8="Push",F8,IF(I8="Loss",0,0)))</f>
         <v>0</v>
       </c>
-      <c r="K8" s="91" t="n">
+      <c r="K8" s="39" t="n">
         <f aca="false">IF(I8="Pending",0,J8-F8)</f>
         <v>0</v>
       </c>
-      <c r="L8" s="70" t="n">
+      <c r="L8" s="69" t="n">
         <v>0.54</v>
       </c>
       <c r="M8" s="58" t="s">
         <v>482</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="29" t="n">
         <v>3</v>
       </c>
@@ -3913,66 +3850,66 @@
       <c r="E9" s="35" t="n">
         <v>263</v>
       </c>
-      <c r="F9" s="89" t="n">
+      <c r="F9" s="36" t="n">
         <v>60</v>
       </c>
-      <c r="G9" s="90" t="n">
+      <c r="G9" s="37" t="n">
         <f aca="false">IF(E9&gt;0,F9*E9/100,F9*100/ABS(E9))</f>
         <v>157.8</v>
       </c>
-      <c r="H9" s="90" t="n">
+      <c r="H9" s="37" t="n">
         <f aca="false">F9+G9</f>
         <v>217.8</v>
       </c>
       <c r="I9" s="53" t="s">
         <v>121</v>
       </c>
-      <c r="J9" s="90" t="n">
+      <c r="J9" s="37" t="n">
         <f aca="false">IF(I9="Win",F9+G9,IF(I9="Push",F9,IF(I9="Loss",0,0)))</f>
         <v>0</v>
       </c>
-      <c r="K9" s="91" t="n">
+      <c r="K9" s="39" t="n">
         <f aca="false">IF(I9="Pending",0,J9-F9)</f>
         <v>0</v>
       </c>
-      <c r="L9" s="70" t="n">
+      <c r="L9" s="69" t="n">
         <v>0.32</v>
       </c>
       <c r="M9" s="58" t="s">
         <v>485</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="88" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="4" t="s">
         <v>425</v>
       </c>
-      <c r="F10" s="92" t="n">
+      <c r="F10" s="8" t="n">
         <f aca="false">SUM(F7:F9)</f>
         <v>550</v>
       </c>
-      <c r="G10" s="92" t="n">
+      <c r="G10" s="8" t="n">
         <f aca="false">SUM(G7:G9)</f>
         <v>600.469942669943</v>
       </c>
-      <c r="H10" s="92" t="n">
+      <c r="H10" s="8" t="n">
         <f aca="false">SUM(H7:H9)</f>
         <v>1150.46994266994</v>
       </c>
-      <c r="J10" s="92" t="n">
+      <c r="J10" s="8" t="n">
         <f aca="false">SUM(J7:J9)</f>
         <v>0</v>
       </c>
-      <c r="K10" s="92" t="n">
+      <c r="K10" s="8" t="n">
         <f aca="false">SUM(K7:K9)</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="K7:K10">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>AND(ISNUMBER(K7),K7&gt;0)</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>AND(ISNUMBER(K7),K7&lt;0)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7168,11 +7105,11 @@
         <v>369</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="69" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="68" t="s">
         <v>60</v>
       </c>
-      <c r="B31" s="69" t="s">
+      <c r="B31" s="68" t="s">
         <v>370</v>
       </c>
     </row>
@@ -7896,7 +7833,7 @@
         <f aca="false">IF(I7="Pending",0,J7-F7)</f>
         <v>0</v>
       </c>
-      <c r="L7" s="70" t="n">
+      <c r="L7" s="69" t="n">
         <v>0.18</v>
       </c>
       <c r="M7" s="58" t="s">
@@ -7941,7 +7878,7 @@
         <f aca="false">IF(I8="Pending",0,J8-F8)</f>
         <v>0</v>
       </c>
-      <c r="L8" s="70" t="n">
+      <c r="L8" s="69" t="n">
         <v>0.07</v>
       </c>
       <c r="M8" s="58" t="s">
@@ -7986,7 +7923,7 @@
         <f aca="false">IF(I9="Pending",0,J9-F9)</f>
         <v>0</v>
       </c>
-      <c r="L9" s="70" t="n">
+      <c r="L9" s="69" t="n">
         <v>0.07</v>
       </c>
       <c r="M9" s="58" t="s">
@@ -8031,7 +7968,7 @@
         <f aca="false">IF(I10="Pending",0,J10-F10)</f>
         <v>0</v>
       </c>
-      <c r="L10" s="70" t="n">
+      <c r="L10" s="69" t="n">
         <v>0.055</v>
       </c>
       <c r="M10" s="58" t="s">
@@ -8076,7 +8013,7 @@
         <f aca="false">IF(I11="Pending",0,J11-F11)</f>
         <v>0</v>
       </c>
-      <c r="L11" s="70" t="n">
+      <c r="L11" s="69" t="n">
         <v>0.045</v>
       </c>
       <c r="M11" s="58" t="s">
@@ -8121,7 +8058,7 @@
         <f aca="false">IF(I12="Pending",0,J12-F12)</f>
         <v>0</v>
       </c>
-      <c r="L12" s="70" t="n">
+      <c r="L12" s="69" t="n">
         <v>0.025</v>
       </c>
       <c r="M12" s="58" t="s">
@@ -8129,47 +8066,47 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="71" t="n">
+      <c r="A13" s="70" t="n">
         <v>7</v>
       </c>
-      <c r="B13" s="72" t="s">
+      <c r="B13" s="71" t="s">
         <v>414</v>
       </c>
-      <c r="C13" s="73" t="s">
+      <c r="C13" s="72" t="s">
         <v>415</v>
       </c>
-      <c r="D13" s="71" t="s">
+      <c r="D13" s="70" t="s">
         <v>92</v>
       </c>
-      <c r="E13" s="74" t="n">
+      <c r="E13" s="73" t="n">
         <v>-146</v>
       </c>
-      <c r="F13" s="75" t="n">
+      <c r="F13" s="74" t="n">
         <v>120</v>
       </c>
-      <c r="G13" s="76" t="n">
+      <c r="G13" s="75" t="n">
         <f aca="false">IF(E13&gt;0,F13*E13/100,F13*100/ABS(E13))</f>
         <v>82.1917808219178</v>
       </c>
-      <c r="H13" s="76" t="n">
+      <c r="H13" s="75" t="n">
         <f aca="false">F13+G13</f>
         <v>202.191780821918</v>
       </c>
       <c r="I13" s="53" t="s">
         <v>121</v>
       </c>
-      <c r="J13" s="76" t="n">
+      <c r="J13" s="75" t="n">
         <f aca="false">IF(I13="Win",F13+G13,IF(I13="Push",F13,IF(I13="Loss",0,0)))</f>
         <v>0</v>
       </c>
-      <c r="K13" s="77" t="n">
+      <c r="K13" s="76" t="n">
         <f aca="false">IF(I13="Pending",0,J13-F13)</f>
         <v>0</v>
       </c>
-      <c r="L13" s="78" t="n">
+      <c r="L13" s="77" t="n">
         <v>0.62</v>
       </c>
-      <c r="M13" s="79" t="s">
+      <c r="M13" s="78" t="s">
         <v>416</v>
       </c>
     </row>
@@ -8211,7 +8148,7 @@
         <f aca="false">IF(I14="Pending",0,J14-F14)</f>
         <v>0</v>
       </c>
-      <c r="L14" s="70" t="n">
+      <c r="L14" s="69" t="n">
         <v>0.44</v>
       </c>
       <c r="M14" s="58" t="s">
@@ -8256,7 +8193,7 @@
         <f aca="false">IF(I15="Pending",0,J15-F15)</f>
         <v>0</v>
       </c>
-      <c r="L15" s="70" t="n">
+      <c r="L15" s="69" t="n">
         <v>0.42</v>
       </c>
       <c r="M15" s="58" t="s">
@@ -8301,7 +8238,7 @@
         <f aca="false">IF(I16="Pending",0,J16-F16)</f>
         <v>0</v>
       </c>
-      <c r="L16" s="70" t="n">
+      <c r="L16" s="69" t="n">
         <v>0.42</v>
       </c>
       <c r="M16" s="58" t="s">
@@ -8315,7 +8252,7 @@
       <c r="B17" s="5" t="s">
         <v>423</v>
       </c>
-      <c r="C17" s="80" t="s">
+      <c r="C17" s="79" t="s">
         <v>415</v>
       </c>
       <c r="D17" s="29" t="s">
@@ -8346,7 +8283,7 @@
         <f aca="false">IF(I17="Pending",0,J17-F17)</f>
         <v>0</v>
       </c>
-      <c r="L17" s="70" t="n">
+      <c r="L17" s="69" t="n">
         <v>0.3</v>
       </c>
       <c r="M17" s="58" t="s">
@@ -8354,7 +8291,7 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="81" t="s">
+      <c r="B18" s="80" t="s">
         <v>425</v>
       </c>
       <c r="C18" s="47" t="n">
@@ -8381,7 +8318,7 @@
         <f aca="false">SUM(K7:K17)</f>
         <v>0</v>
       </c>
-      <c r="L18" s="82" t="n">
+      <c r="L18" s="81" t="n">
         <f aca="false">SUM(L7:L17)</f>
         <v>2.645</v>
       </c>
@@ -8512,7 +8449,7 @@
       <c r="A1" s="31" t="s">
         <v>428</v>
       </c>
-      <c r="H1" s="83" t="s">
+      <c r="H1" s="82" t="s">
         <v>429</v>
       </c>
     </row>
@@ -8610,7 +8547,7 @@
         <f aca="false">IF(I7="Pending",0,J7-F7)</f>
         <v>-220</v>
       </c>
-      <c r="L7" s="70" t="n">
+      <c r="L7" s="69" t="n">
         <v>0.27</v>
       </c>
       <c r="M7" s="58" t="s">
@@ -8655,7 +8592,7 @@
         <f aca="false">IF(I8="Pending",0,J8-F8)</f>
         <v>-130</v>
       </c>
-      <c r="L8" s="70" t="n">
+      <c r="L8" s="69" t="n">
         <v>0.18</v>
       </c>
       <c r="M8" s="58" t="s">
@@ -8700,7 +8637,7 @@
         <f aca="false">IF(I9="Pending",0,J9-F9)</f>
         <v>-180</v>
       </c>
-      <c r="L9" s="70" t="n">
+      <c r="L9" s="69" t="n">
         <v>0.6</v>
       </c>
       <c r="M9" s="58" t="s">
@@ -8745,7 +8682,7 @@
         <f aca="false">IF(I10="Pending",0,J10-F10)</f>
         <v>136.363636363636</v>
       </c>
-      <c r="L10" s="70" t="n">
+      <c r="L10" s="69" t="n">
         <v>0.58</v>
       </c>
       <c r="M10" s="58" t="s">
@@ -8790,7 +8727,7 @@
         <f aca="false">IF(I11="Pending",0,J11-F11)</f>
         <v>-120</v>
       </c>
-      <c r="L11" s="70" t="n">
+      <c r="L11" s="69" t="n">
         <v>0.57</v>
       </c>
       <c r="M11" s="58" t="s">
@@ -8835,7 +8772,7 @@
         <f aca="false">IF(I12="Pending",0,J12-F12)</f>
         <v>113.636363636364</v>
       </c>
-      <c r="L12" s="70" t="n">
+      <c r="L12" s="69" t="n">
         <v>0.56</v>
       </c>
       <c r="M12" s="58" t="s">
@@ -8880,7 +8817,7 @@
         <f aca="false">IF(I13="Pending",0,J13-F13)</f>
         <v>-75</v>
       </c>
-      <c r="L13" s="70" t="n">
+      <c r="L13" s="69" t="n">
         <v>0.07</v>
       </c>
       <c r="M13" s="58" t="s">

</xml_diff>

<commit_message>
Open R3 tee sheet official: Herbert leads Suber/Young/Gerard by 2, final twosome Herbert-Suber 10:50 ET (DeChambeau revised out, 10:30 w/ Burns); Koepka thru cut now TWO-SOURCE (4:50 ET tee time, GC+Yahoo); Morikawa CONFIRMED thru cut (PGA Tour + 8:10 ET tee); all 5 surviving outrights play weekend; banner+dashboard+tracker refresh
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AaFwLnfuCnYkoSz9rho6NS
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -7801,9 +7801,9 @@
           <t>TEST 6 — THE 154th OPEN CHAMPIONSHIP · ROYAL BIRKDALE · JULY 16-19, 2026</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>STATUS: ACTIVE — R2 COMPLETE Fri Jul 17 (11:08 PM UK): Herbert −8 leads; Sat final pairing Herbert/DeChambeau (−7) official per Yahoo. Our card: Scheffler −4 four back (2-source); Rahm −4, Fleetwood −3 (GM; Yahoo has both in Sat last groups); cut +1 — Fitzpatrick +4 MISSED CUT ($150 dead). NEW: Koepka MADE CUT per Yahoo (single-source) — +5000 longshot alive. Morikawa unconfirmed. Grades Sunday.</t>
+      <c r="B1" s="85" t="inlineStr">
+        <is>
+          <t>STATUS: ACTIVE — R3 TEE SHEET OFFICIAL Sat Jul 18 (3:08 AM UK): Herbert −8 leads Suber/Young/Gerard by 2 (Golf Channel verbatim); final twosome Herbert–Suber 10:50 ET — DeChambeau revised out of final pairing (10:30 w/ Burns). Our card: Scheffler −4 tees 9:45 ET; Rahm &amp; Fleetwood paired 9:35 ET; Fitzpatrick +4 MISSED CUT ($150 dead). Koepka thru cut TWO-SOURCE (4:50 ET tee time, GC+Yahoo) — +5000 alive. Morikawa CONFIRMED thru cut (PGA Tour + 8:10 ET tee time). All 5 surviving outrights play weekend. Grades Sunday.</t>
         </is>
       </c>
       <c r="H1" s="137" t="inlineStr">

</xml_diff>

<commit_message>
Hourly refresh: Open R3 banner 4:10 PM UK — Fox in clubhouse at -8, Herbert on course; Koepka +1 nine back
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015L9Ai9EktdySrFvpXUWcnc
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -1229,10 +1229,10 @@
     <t xml:space="preserve">TEST 6 — THE 154th OPEN CHAMPIONSHIP · ROYAL BIRKDALE · JULY 16-19, 2026</t>
   </si>
   <si>
+    <t xml:space="preserve">STATUS: ACTIVE — R3 MID-ROUND Sat Jul 18 (4:10 PM UK): Ryan Fox IN THE CLUBHOUSE at −8 after a record-tying 62 (nine birdies, one bogey) — shares the lead with Herbert −8, who teed off 3:50 PM UK (Central Oregon Daily + Golfmagic live boards agree). Suber/Young −6; DeChambeau −5. Our card: Scheffler/Rahm/Fleetwood all −4 (T10), an hour into Moving Day; JT also −4; Morikawa −2; Koepka +1 — nine back, +5000 on life support. Fitzpatrick MC $150 dead. Grades Sunday only.</t>
+  </si>
+  <si>
     <t xml:space="preserve">STATUS: ACTIVE — R3 MID-ROUND Sat Jul 18 (3:10 PM UK): Ryan Fox posts a record-tying 62 (nine birdies, one bogey) — now −8 with a SHARE OF THE LEAD; Herbert −8 tees off 3:50 PM UK (Yahoo Sports + Central Oregon Daily live board agree). DeChambeau −5. Our card: Scheffler/Rahm/Fleetwood all −4 (T10), just teed off 2:35–2:45 PM UK; JT also −4 thru 10; Morikawa and Koepka outside the live top 10 — Koepka +5000 needs a big weekend. Fitzpatrick MC $150 dead. Grades Sunday only.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STATUS: ACTIVE — R2 COMPLETE Fri Jul 17 (10:20 PM UK): Herbert −8 leads (70-62); DeChambeau −7 solo 2nd after 2-stroke penalty; Suber/Young −6, Burns −5. Our card: Scheffler −4 four back (2-source); Rahm −4, Fleetwood −3 (GM, single-source); cut +1 — Fitzpatrick +4 MISSED CUT ($150 dead). Morikawa/Koepka unconfirmed. Grades Sunday.</t>
   </si>
   <si>
     <t xml:space="preserve">Source: open2026-betting-card.html · Outrights locked Sun Jul 12 · Phase 2 top-10 props deployed Wed Jul 15 (reserved $400 now at risk)</t>

</xml_diff>

<commit_message>
Hourly refresh: Open R3 banner 7:30 PM UK — four-way tie at -8 (Fox 62/Herbert/Burns/Si Woo); Fleetwood charging -6/-7 within two; Scheffler -5, Rahm ~-3/-4; nothing grades until Sunday
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K93LfP4v6b2WnaTYHbYjfv
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="486">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="487">
   <si>
     <t xml:space="preserve">BETTING TEST ACCOUNT — ROLL-UP DASHBOARD</t>
   </si>
@@ -1227,6 +1227,9 @@
   </si>
   <si>
     <t xml:space="preserve">TEST 6 — THE 154th OPEN CHAMPIONSHIP · ROYAL BIRKDALE · JULY 16-19, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STATUS: ACTIVE — R3 LATE Sat Jul 18 (7:30 PM UK): four-way tie at −8 — Fox (record-tying 62, in the clubhouse), Herbert, Burns (touched −9 before a bogey at 9) and Si Woo Kim (Golf Monthly liveblog 5:33 PM UK + Central Oregon Daily liveblog agree; feeds lag the course ~1-2h). Young −7. OUR CARD: Fleetwood finally moving — birdies at 5, 7 and 11 have him −6/−7 and within two (PGA Tour calls it a 'storybook run'); Scheffler grinding at −5; Rahm flat around −3/−4; no R3 move reported for Morikawa (−2 start) or Koepka (+1 start — +5000 still on life support). Fitzpatrick MC $150 dead. Grades Sunday only.</t>
   </si>
   <si>
     <t xml:space="preserve">STATUS: ACTIVE — R3 MID-ROUND Sat Jul 18 (6:15 PM UK): Fox in the clubhouse at −8 (record-tying 62) and Herbert −8 still share the lead (Central Oregon Daily liveblog 1:27 PM ET + Golf Channel liveblog agree). Chase: Suber/Young/Gerard −6; Burns/DeChambeau/Si Woo Kim −5. Our card: Scheffler/Rahm/Fleetwood all −4 (T10) mid-round; JT −4 thru 9; Schauffele in at −4 (66); Morikawa −2; Koepka +1 — nine back, +5000 on life support. Fitzpatrick MC $150 dead. Grades Sunday only.</t>
@@ -3230,20 +3233,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="31" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="H1" s="83" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3297,10 +3300,10 @@
         <v>1</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="D7" s="29" t="s">
         <v>377</v>
@@ -3334,7 +3337,7 @@
         <v>0.57</v>
       </c>
       <c r="M7" s="58" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3342,10 +3345,10 @@
         <v>2</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D8" s="29" t="s">
         <v>177</v>
@@ -3379,7 +3382,7 @@
         <v>0.54</v>
       </c>
       <c r="M8" s="58" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3387,10 +3390,10 @@
         <v>3</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C9" s="28" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="D9" s="29" t="s">
         <v>177</v>
@@ -3424,7 +3427,7 @@
         <v>0.55</v>
       </c>
       <c r="M9" s="58" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3432,7 +3435,7 @@
         <v>4</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C10" s="28" t="s">
         <v>392</v>
@@ -3469,7 +3472,7 @@
         <v>0.54</v>
       </c>
       <c r="M10" s="58" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3477,10 +3480,10 @@
         <v>5</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="C11" s="28" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="D11" s="29" t="s">
         <v>87</v>
@@ -3514,7 +3517,7 @@
         <v>0.58</v>
       </c>
       <c r="M11" s="58" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3522,10 +3525,10 @@
         <v>6</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="C12" s="28" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="D12" s="29" t="s">
         <v>377</v>
@@ -3559,7 +3562,7 @@
         <v>0.52</v>
       </c>
       <c r="M12" s="58" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3570,7 +3573,7 @@
         <v>394</v>
       </c>
       <c r="C13" s="28" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="D13" s="29" t="s">
         <v>115</v>
@@ -3604,7 +3607,7 @@
         <v>0.1</v>
       </c>
       <c r="M13" s="58" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3682,20 +3685,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="31" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="H1" s="84" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3749,13 +3752,13 @@
         <v>1</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="D7" s="29" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="E7" s="35" t="n">
         <v>-111</v>
@@ -3786,7 +3789,7 @@
         <v>0.6</v>
       </c>
       <c r="M7" s="58" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3794,13 +3797,13 @@
         <v>2</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="D8" s="29" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="E8" s="35" t="n">
         <v>-110</v>
@@ -3831,7 +3834,7 @@
         <v>0.54</v>
       </c>
       <c r="M8" s="58" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3839,10 +3842,10 @@
         <v>3</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="C9" s="28" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="D9" s="29" t="s">
         <v>115</v>
@@ -3876,12 +3879,12 @@
         <v>0.32</v>
       </c>
       <c r="M9" s="58" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="4" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="F10" s="8" t="n">
         <f aca="false">SUM(F7:F9)</f>
@@ -7739,17 +7742,17 @@
         <v>399</v>
       </c>
       <c r="H1" s="52" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7803,7 +7806,7 @@
         <v>1</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C7" s="28" t="s">
         <v>285</v>
@@ -7840,7 +7843,7 @@
         <v>0.18</v>
       </c>
       <c r="M7" s="58" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7848,7 +7851,7 @@
         <v>2</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C8" s="28" t="s">
         <v>285</v>
@@ -7885,7 +7888,7 @@
         <v>0.07</v>
       </c>
       <c r="M8" s="58" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7893,7 +7896,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C9" s="28" t="s">
         <v>285</v>
@@ -7930,7 +7933,7 @@
         <v>0.07</v>
       </c>
       <c r="M9" s="58" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7938,7 +7941,7 @@
         <v>4</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C10" s="28" t="s">
         <v>285</v>
@@ -7975,7 +7978,7 @@
         <v>0.055</v>
       </c>
       <c r="M10" s="58" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7983,7 +7986,7 @@
         <v>5</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C11" s="28" t="s">
         <v>285</v>
@@ -8020,7 +8023,7 @@
         <v>0.045</v>
       </c>
       <c r="M11" s="58" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8028,7 +8031,7 @@
         <v>6</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C12" s="28" t="s">
         <v>285</v>
@@ -8065,7 +8068,7 @@
         <v>0.025</v>
       </c>
       <c r="M12" s="58" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8073,10 +8076,10 @@
         <v>7</v>
       </c>
       <c r="B13" s="71" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C13" s="72" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D13" s="70" t="s">
         <v>92</v>
@@ -8110,7 +8113,7 @@
         <v>0.62</v>
       </c>
       <c r="M13" s="78" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8118,10 +8121,10 @@
         <v>8</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C14" s="28" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D14" s="29" t="s">
         <v>92</v>
@@ -8155,7 +8158,7 @@
         <v>0.44</v>
       </c>
       <c r="M14" s="58" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8163,10 +8166,10 @@
         <v>9</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C15" s="28" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D15" s="29" t="s">
         <v>92</v>
@@ -8200,7 +8203,7 @@
         <v>0.42</v>
       </c>
       <c r="M15" s="58" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8208,10 +8211,10 @@
         <v>10</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C16" s="28" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D16" s="29" t="s">
         <v>92</v>
@@ -8245,7 +8248,7 @@
         <v>0.42</v>
       </c>
       <c r="M16" s="58" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8253,10 +8256,10 @@
         <v>11</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C17" s="79" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D17" s="29" t="s">
         <v>92</v>
@@ -8290,12 +8293,12 @@
         <v>0.3</v>
       </c>
       <c r="M17" s="58" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="80" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="C18" s="47" t="n">
         <f aca="false">COUNTIF(I7:I12,"Loss")</f>
@@ -8346,7 +8349,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="5" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C21" s="30" t="n">
         <f aca="false">SUM(F7:F12)</f>
@@ -8373,7 +8376,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="5" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C24" s="48" t="n">
         <f aca="false">SUM(L7:L12)</f>
@@ -8450,20 +8453,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="31" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="H1" s="82" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8517,7 +8520,7 @@
         <v>1</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C7" s="28" t="s">
         <v>285</v>
@@ -8554,7 +8557,7 @@
         <v>0.27</v>
       </c>
       <c r="M7" s="58" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8562,7 +8565,7 @@
         <v>2</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C8" s="28" t="s">
         <v>285</v>
@@ -8599,7 +8602,7 @@
         <v>0.18</v>
       </c>
       <c r="M8" s="58" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8607,10 +8610,10 @@
         <v>3</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C9" s="28" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="D9" s="29" t="s">
         <v>92</v>
@@ -8644,7 +8647,7 @@
         <v>0.6</v>
       </c>
       <c r="M9" s="58" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8652,10 +8655,10 @@
         <v>4</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="C10" s="28" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D10" s="29" t="s">
         <v>92</v>
@@ -8689,7 +8692,7 @@
         <v>0.58</v>
       </c>
       <c r="M10" s="58" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8697,10 +8700,10 @@
         <v>5</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C11" s="28" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="D11" s="29" t="s">
         <v>92</v>
@@ -8734,7 +8737,7 @@
         <v>0.57</v>
       </c>
       <c r="M11" s="58" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8742,10 +8745,10 @@
         <v>6</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C12" s="28" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D12" s="29" t="s">
         <v>92</v>
@@ -8779,7 +8782,7 @@
         <v>0.56</v>
       </c>
       <c r="M12" s="58" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8787,7 +8790,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C13" s="28" t="s">
         <v>285</v>
@@ -8824,7 +8827,7 @@
         <v>0.07</v>
       </c>
       <c r="M13" s="58" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Hourly refresh: OPEN R3 leaderboard CORRECTED — Burns' Saturday 65 ties Herbert for lead at -9, Fox's 62 one back (PGA Tour + Golf Channel + NBC headlines agree); prior 'final board -8 / our guys -4' read was a stale 36-hole block. RUGBY live: USA 14-7 Spain near half — USA -3.5 + parlay leg 2 pending, grades at FT. No bets graded; no balance change. Banners/tracker/PDFs updated.
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L682xyPTFma2D96wLpdv3g
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -1229,7 +1229,7 @@
     <t xml:space="preserve">TEST 6 — THE 154th OPEN CHAMPIONSHIP · ROYAL BIRKDALE · JULY 16-19, 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">STATUS: ACTIVE — R3 LATE Sat Jul 18 (8:15 PM UK): Fox pars 18 for a record-tying 62 — clubhouse co-lead with Herbert at −8; Burns &amp; Si Woo Kim slip back ~−5/−6 into the Suber/Young/Gerard chase pack (~−6). OUR CARD: Fleetwood −7 thru 13 on last full board — one-two back; Scheffler ~−4/−5; Rahm ~−3/−4; Morikawa −2; Koepka +1. Grades Sunday only. (Central Oregon Daily + PGA Tour liveblogs agree)</t>
+    <t xml:space="preserve">STATUS: ACTIVE — R3 COMPLETE, CORRECTED (Sat ~7:45 PM CT): PGA Tour + Golf Channel + NBC end-of-day headlines agree — Sam Burns’ Saturday 65 grabs a share of the lead with Lucas Herbert at −9; Ryan Fox’s 62 (posted −8 F) one back. Earlier "Fox &amp; Herbert co-lead −8 / our guys −4" read came from a stale 36-hole block — superseded. OUR CARD: Fleetwood finished in the chase pack (was −7 thru 13 on last in-round board); Scheffler/Rahm mid-single digits; Morikawa ~−2; Koepka ~+1, ten back. Re-verify exact 54-hole numbers from final board before Sunday grading. Grades Sunday only.</t>
   </si>
   <si>
     <t xml:space="preserve">Source: open2026-betting-card.html · Outrights locked Sun Jul 12 · Phase 2 top-10 props deployed Wed Jul 15 (reserved $400 now at risk)</t>
@@ -1451,7 +1451,7 @@
     <t xml:space="preserve">TEST 7 — WORLD RUGBY NATIONS CUP · FINAL ROUND · JULY 18, 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">STATUS: ACTIVE — Georgia leg WON (49-22); USA-Spain ~6:30 PM CT decides card</t>
+    <t xml:space="preserve">STATUS: ACTIVE — Georgia leg WON (49-22); USA-Spain LIVE: USA 14-7 near halftime (RugbyPass, ~7:15 PM CT check); grades at full time</t>
   </si>
   <si>
     <t xml:space="preserve">Source: cards/rugby-jul18-betting-card.html · Lines: freetips.com / Stake.com handicaps, finalized Fri Jul 17</t>

</xml_diff>

<commit_message>
Hourly refresh: RUGBY CARD SETTLED 3-for-3 — USA 29-22 Spain FT (Sky Sports + UltimateRugby agree), USA -3.5 covered by 3.5; +263 longshot parlay HIT (first of the test, 1-for-7). Card +$600.47, balance $3,544.15 (-29.1%). Betty settle clip + greeting regenerated; card archived on index; dashboard tiles/timeline/slots/longshot tracker + PDFs updated. The Open (last active card) grades Sunday evening.
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -1451,7 +1451,7 @@
     <t xml:space="preserve">TEST 7 — WORLD RUGBY NATIONS CUP · FINAL ROUND · JULY 18, 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">STATUS: ACTIVE — Georgia leg WON (49-22); USA-Spain LIVE: USA 14-7 near halftime (RugbyPass, ~7:15 PM CT check); grades at full time</t>
+    <t xml:space="preserve">STATUS: SETTLED — swept the card 3-for-3: Georgia 49-22 Chile, USA 29-22 Spain; LONGSHOT parlay (+263) HIT. Card +$600.47</t>
   </si>
   <si>
     <t xml:space="preserve">Source: cards/rugby-jul18-betting-card.html · Lines: freetips.com / Stake.com handicaps, finalized Fri Jul 17</t>
@@ -1478,7 +1478,7 @@
     <t xml:space="preserve">USA vs Spain · ~6:30 PM CT</t>
   </si>
   <si>
-    <t xml:space="preserve">Centerpiece — USA 2-0, backed to cover vs inconsistent Spain</t>
+    <t xml:space="preserve">Centerpiece — USA 2-0, backed to cover vs inconsistent Spain · GRADED Sat Jul 18: USA 29-22 Spain (FT, won by 7, covered -3.5) — Sky Sports + UltimateRugby agree</t>
   </si>
   <si>
     <t xml:space="preserve">LONGSHOT: Georgia -12.5 + USA -3.5</t>
@@ -1487,7 +1487,7 @@
     <t xml:space="preserve">2-leg cross-match parlay</t>
   </si>
   <si>
-    <t xml:space="preserve">Round's longshot (modest — only 2 markets priced); counts in longshot record · Leg 1 (Georgia -12.5) WON 49-22; rides on USA -3.5</t>
+    <t xml:space="preserve">Round's longshot (modest — only 2 markets priced); counts in longshot record · Leg 1 (Georgia -12.5) WON 49-22; rides on USA -3.5 · GRADED Sat Jul 18: Leg 2 (USA -3.5) WON 29-22 — PARLAY HITS at +263, first longshot HIT of the test</t>
   </si>
 </sst>
 </file>
@@ -2478,7 +2478,7 @@
       </c>
       <c r="B6" s="7" t="n">
         <f aca="false">H25</f>
-        <v>-1750.01031855575</v>
+        <v>-1455.84668219211</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">B5+B6</f>
-        <v>3249.98968144425</v>
+        <v>3544.15331780789</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2496,7 +2496,7 @@
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">F25</f>
-        <v>1210</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">B7-B8</f>
-        <v>2039.98968144425</v>
+        <v>2544.15331780789</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="B10" s="10" t="str">
         <f aca="false">COUNTIF(D16:D24,"ACTIVE")&amp;" of 4 max"</f>
-        <v>2 of 4 max</v>
+        <v>1 of 4 max</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2670,33 +2670,33 @@
       <c r="M18" s="1"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="20" t="n">
+      <c r="A19" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="B19" s="21" t="s">
+      <c r="B19" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="C19" s="20" t="s">
+      <c r="C19" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="D19" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="E19" s="23" t="n">
+      <c r="D19" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="E19" s="17" t="n">
         <f aca="false">SUM('Rugby Jul 18'!F7:F9)</f>
         <v>550</v>
       </c>
-      <c r="F19" s="23" t="n">
+      <c r="F19" s="17" t="n">
         <f aca="false">SUMIF('Rugby Jul 18'!I7:I9,"Pending",'Rugby Jul 18'!F7:F9)</f>
-        <v>210</v>
-      </c>
-      <c r="G19" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="17" t="n">
         <f aca="false">SUM('Rugby Jul 18'!J7:J9)</f>
-        <v>646.306306306306</v>
-      </c>
-      <c r="H19" s="23" t="n">
+        <v>1150.46994266994</v>
+      </c>
+      <c r="H19" s="17" t="n">
         <f aca="false">SUM('Rugby Jul 18'!K7:K9)</f>
-        <v>306.306306306306</v>
+        <v>600.469942669943</v>
       </c>
       <c r="I19" s="18"/>
       <c r="J19" s="19"/>
@@ -2888,15 +2888,15 @@
       </c>
       <c r="F25" s="8" t="n">
         <f aca="false">SUM(F16:F24)</f>
-        <v>1210</v>
+        <v>1000</v>
       </c>
       <c r="G25" s="8" t="n">
         <f aca="false">SUM(G16:G24)</f>
-        <v>5639.98968144425</v>
+        <v>6144.15331780789</v>
       </c>
       <c r="H25" s="8" t="n">
         <f aca="false">SUM(H16:H24)</f>
-        <v>-1750.01031855575</v>
+        <v>-1455.84668219211</v>
       </c>
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
@@ -3063,7 +3063,7 @@
       </c>
       <c r="E34" s="10" t="str">
         <f aca="false">IF('Rugby Jul 18'!I9="Win","HIT",IF('Rugby Jul 18'!I9="Loss","MISS","Pending"))</f>
-        <v>Pending</v>
+        <v>HIT</v>
       </c>
       <c r="K34" s="1"/>
       <c r="L34" s="1"/>
@@ -3117,7 +3117,7 @@
       </c>
       <c r="E37" s="10" t="str">
         <f aca="false">IF(COUNTIF(E29:E36,"HIT")+COUNTIF(E29:E36,"MISS")=0,"—",COUNTIF(E29:E36,"HIT")&amp;"-for-"&amp;(COUNTIF(E29:E36,"HIT")+COUNTIF(E29:E36,"MISS"))&amp;" ("&amp;TEXT(COUNTIF(E29:E36,"HIT")/(COUNTIF(E29:E36,"HIT")+COUNTIF(E29:E36,"MISS")),"0%")&amp;")")</f>
-        <v>0-for-6 (0%)</v>
+        <v>1-for-7 (14%)</v>
       </c>
       <c r="K37" s="1"/>
       <c r="L37" s="1"/>
@@ -3817,15 +3817,15 @@
         <v>286.363636363636</v>
       </c>
       <c r="I8" s="53" t="s">
-        <v>121</v>
+        <v>88</v>
       </c>
       <c r="J8" s="37" t="n">
         <f aca="false">IF(I8="Win",F8+G8,IF(I8="Push",F8,IF(I8="Loss",0,0)))</f>
-        <v>0</v>
+        <v>286.363636363636</v>
       </c>
       <c r="K8" s="39" t="n">
         <f aca="false">IF(I8="Pending",0,J8-F8)</f>
-        <v>0</v>
+        <v>136.363636363636</v>
       </c>
       <c r="L8" s="69" t="n">
         <v>0.54</v>
@@ -3862,15 +3862,15 @@
         <v>217.8</v>
       </c>
       <c r="I9" s="53" t="s">
-        <v>121</v>
+        <v>88</v>
       </c>
       <c r="J9" s="37" t="n">
         <f aca="false">IF(I9="Win",F9+G9,IF(I9="Push",F9,IF(I9="Loss",0,0)))</f>
-        <v>0</v>
+        <v>217.8</v>
       </c>
       <c r="K9" s="39" t="n">
         <f aca="false">IF(I9="Pending",0,J9-F9)</f>
-        <v>0</v>
+        <v>157.8</v>
       </c>
       <c r="L9" s="69" t="n">
         <v>0.32</v>
@@ -3897,11 +3897,11 @@
       </c>
       <c r="J10" s="8" t="n">
         <f aca="false">SUM(J7:J9)</f>
-        <v>646.306306306306</v>
+        <v>1150.46994266994</v>
       </c>
       <c r="K10" s="8" t="n">
         <f aca="false">SUM(K7:K9)</f>
-        <v>306.306306306306</v>
+        <v>600.469942669943</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
The Open SETTLES 2-9 (-$565.61): Rahm T46 + Morikawa T18 miss the top-10, final props lose (verified GolfNewsNet + Yahoo payout boards) — board clean, all July cards settled; balance $2,978.55 (-40.4%); Betty settle + fresh greeting
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015YMUm4y8QbG8yBTprjVfWw
</commit_message>
<xml_diff>
--- a/betting_tracker.xlsx
+++ b/betting_tracker.xlsx
@@ -206,7 +206,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -291,6 +291,12 @@
         <bgColor rgb="FF993366"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE7E6E6"/>
+        <bgColor rgb="FFE7E6E6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -326,7 +332,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="170">
+  <cellXfs count="171">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -834,6 +840,9 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1383,9 +1392,9 @@
           <t>Jul 16-19</t>
         </is>
       </c>
-      <c r="D18" s="107" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+      <c r="D18" s="170" t="inlineStr">
+        <is>
+          <t>SETTLED</t>
         </is>
       </c>
       <c r="E18" s="108">
@@ -7798,24 +7807,12 @@
     <row r="1" ht="15.75" customHeight="1" s="86">
       <c r="A1" s="116" t="inlineStr">
         <is>
-          <t>STATUS: ACTIVE — 9 of 11 GRADED (Sun Jul 19 eve): Ryan Fox birdies the 72nd to win at −10 (Young −9, Burns −8) — all six outrights LOSE, Koepka LONGSHOT MISS (0-for-6); Scheffler + Fleetwood top-10s CASH (both T4 −7), Fitzpatrick top-10 dead (MC); card −$445.61 so far with Rahm + Morikawa top-10 props ($120) awaiting full final board — settles next run</t>
-        </is>
-      </c>
-      <c r="B1" s="85" t="inlineStr">
-        <is>
-          <t>STATUS: ACTIVE — FINAL ROUND LIVE (Sun ~12:10 PM CT; Golf Monthly ~5:21 PM local): Si Woo Kim leads at −10 deep into the back nine, still bettering the clubhouse target; Cameron Young clubhouse −9 (64); Sam Burns has stumbled to −8 alongside Ryan Fox in the final group as the wind gets up; Scheffler −7 thru 16, Fleetwood and Herbert −7 — outrights need a leader collapse, Scheffler/Fleetwood top-10 props look strong; grades tonight off verified final board</t>
-        </is>
-      </c>
-      <c r="H1" s="137" t="inlineStr">
-        <is>
-          <t>STATUS: ACTIVE — FINAL ROUND LIVE (Sun ~12:10 PM CT; Golf Monthly ~5:21 PM local): Si Woo Kim leads at −10 deep into the back nine, still bettering the clubhouse target; Cameron Young clubhouse −9 (64); Sam Burns has stumbled to −8 alongside Ryan Fox in the final group as the wind gets up; Scheffler −7 thru 16, Fleetwood and Herbert −7 — outrights need a leader collapse, Scheffler/Fleetwood top-10 props look strong; grades tonight off verified final board</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>STATUS: ACTIVE — 9 of 11 GRADED (Sun Jul 19 eve): Ryan Fox birdies the 72nd to win at −10 (Young −9, Burns −8) — all six outrights LOSE, Koepka LONGSHOT MISS (0-for-6); Scheffler + Fleetwood top-10s CASH (both T4 −7), Fitzpatrick top-10 dead (MC); card −$445.61 so far with Rahm + Morikawa top-10 props ($120) awaiting full final board — settles next run</t>
-        </is>
-      </c>
+          <t>STATUS: SETTLED (Sun Jul 19 night): Ryan Fox birdies the 72nd to win at −10 (Young −9, Burns −8) — all six outrights LOSE, Koepka LONGSHOT MISS (0-for-6); Scheffler + Fleetwood top-10s CASH (both T4 −7); Rahm (T46, E) and Morikawa (T18, −3) both miss the top-10 — final props LOSE. Card settles −$565.61 on $1,000 staked (returned $434.39). Verified: GolfNewsNet + Yahoo payouts final boards agree.</t>
+        </is>
+      </c>
+      <c r="B1" s="85" t="n"/>
+      <c r="H1" s="137" t="n"/>
+      <c r="I1" s="85" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1" s="86">
       <c r="A2" s="88" t="inlineStr">
@@ -8380,7 +8377,7 @@
       </c>
       <c r="I15" s="138" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Loss</t>
         </is>
       </c>
       <c r="J15" s="122">
@@ -8490,7 +8487,7 @@
       </c>
       <c r="I17" s="138" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Loss</t>
         </is>
       </c>
       <c r="J17" s="122">

</xml_diff>